<commit_message>
MAJ des pdf manquants
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\d-diperi\Desktop\fo-ico-documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2618AAED-CDE1-4EB6-8254-5B0900CED5D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C50DD1-50C5-421B-B80A-12206A0A6665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="138">
   <si>
     <t>Catégorie</t>
   </si>
@@ -165,12 +165,6 @@
     <t>Forfait Mobilité Durable</t>
   </si>
   <si>
-    <t>24/10/2025</t>
-  </si>
-  <si>
-    <t>⚠️ À vérifier : lors d'un contrôle précédent, le PDF présent semblait être la version 2024, pas 2025 — à recontrôler sur ce nouvel export</t>
-  </si>
-  <si>
     <t>Intéressement 2024</t>
   </si>
   <si>
@@ -201,9 +195,6 @@
     <t>30/06/2021</t>
   </si>
   <si>
-    <t>Pas de PDF ; accord de base (30/01/2020) absent du dépôt</t>
-  </si>
-  <si>
     <t>Intergénérationnel — avenant 2023</t>
   </si>
   <si>
@@ -261,18 +252,12 @@
     <t>Supplément d'intéressement 2023</t>
   </si>
   <si>
-    <t>Pas de PDF pour l'exercice 2023 spécifiquement</t>
-  </si>
-  <si>
     <t>Supplément d'intéressement 2025</t>
   </si>
   <si>
     <t>17/04/2026</t>
   </si>
   <si>
-    <t>Converti depuis la dernière mise à jour du dépôt</t>
-  </si>
-  <si>
     <t>Travail de nuit 2026</t>
   </si>
   <si>
@@ -384,9 +369,6 @@
     <t>non identifiée</t>
   </si>
   <si>
-    <t>Converti par OCR (PDF scanné), pas depuis un Word ; aucun bloc de signature trouvé dans le texte</t>
-  </si>
-  <si>
     <t>Élections</t>
   </si>
   <si>
@@ -396,9 +378,6 @@
     <t>12/10/2022</t>
   </si>
   <si>
-    <t>Pas de PDF repéré à cet emplacement</t>
-  </si>
-  <si>
     <t>Vote électronique 2026</t>
   </si>
   <si>
@@ -420,9 +399,6 @@
     <t>PAPE 2022 (préparatoire)</t>
   </si>
   <si>
-    <t>Abandonné/obsolète — exclu volontairement de la conversion</t>
-  </si>
-  <si>
     <t>CCN</t>
   </si>
   <si>
@@ -472,13 +448,31 @@
   </si>
   <si>
     <t>Note : tableau construit en téléchargeant l'archive complète du dépôt GitHub (codeload.github.com) et en inspectant chaque dossier/fichier directement — pas une reconstitution de mémoire. « Word » signifie qu'un fichier .docx correspondant existe dans un sous-dossier « Format word » du dépôt.</t>
+  </si>
+  <si>
+    <t>plus en vigueur</t>
+  </si>
+  <si>
+    <r>
+      <t>⚠️ À vérifier : lors d'un contrôle précédent, le PDF présent semblait être la version 2024, pas 2025 — à recontrôler sur ce nouvel export</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> la date de l'accord est le 26/04/2024</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -537,8 +531,22 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -557,8 +565,26 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -581,11 +607,91 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalDown="1">
+      <left style="thin">
+        <color rgb="FFD0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D5DD"/>
+      </bottom>
+      <diagonal style="thin">
+        <color indexed="64"/>
+      </diagonal>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D5DD"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D5DD"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D5DD"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D5DD"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD0D5DD"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -626,6 +732,44 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -923,168 +1067,176 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="36" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="33">
+        <v>45408</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="30" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="26" customFormat="1" ht="24" x14ac:dyDescent="0.35">
+      <c r="A3" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>11</v>
-      </c>
       <c r="F3" s="12" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>15</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="8"/>
+      <c r="A4" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>18</v>
+        <v>116</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="32" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="13"/>
+      <c r="G5" s="13" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="8"/>
+      <c r="A6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>22</v>
+        <v>112</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="19" t="s">
         <v>11</v>
       </c>
       <c r="G7" s="13" t="s">
-        <v>24</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>7</v>
+        <v>119</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>11</v>
+        <v>47</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>10</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="8"/>
+      <c r="G8" s="8" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>27</v>
+        <v>91</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>28</v>
+        <v>92</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>10</v>
@@ -1096,18 +1248,18 @@
         <v>11</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>24</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>10</v>
@@ -1119,39 +1271,41 @@
         <v>11</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="13"/>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="24" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>11</v>
@@ -1162,17 +1316,19 @@
       <c r="F12" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="8" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>34</v>
+        <v>86</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>11</v>
@@ -1183,41 +1339,45 @@
       <c r="F13" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="8"/>
+      <c r="G13" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="24" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
         <v>7</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>10</v>
+        <v>14</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E15" s="12" t="s">
         <v>11</v>
@@ -1226,18 +1386,18 @@
         <v>11</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="24" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>11</v>
@@ -1249,7 +1409,7 @@
         <v>11</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
@@ -1257,10 +1417,10 @@
         <v>7</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>11</v>
@@ -1271,17 +1431,19 @@
       <c r="F17" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="13"/>
+      <c r="G17" s="13" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>11</v>
@@ -1292,50 +1454,54 @@
       <c r="F18" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="8"/>
+      <c r="G18" s="8" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="13"/>
+      <c r="A19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>50</v>
+      <c r="A20" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
@@ -1343,13 +1509,13 @@
         <v>7</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>10</v>
+        <v>28</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>11</v>
       </c>
       <c r="E21" s="12" t="s">
         <v>11</v>
@@ -1358,7 +1524,7 @@
         <v>11</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
@@ -1366,10 +1532,10 @@
         <v>7</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>11</v>
@@ -1380,94 +1546,100 @@
       <c r="F22" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G22" s="8"/>
+      <c r="G22" s="8" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>58</v>
+      <c r="A23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="8"/>
+      <c r="A24" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="13"/>
+      <c r="A25" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" s="29" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>24</v>
+      <c r="A26" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
@@ -1475,13 +1647,13 @@
         <v>7</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>11</v>
+        <v>42</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>10</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>11</v>
@@ -1489,19 +1661,21 @@
       <c r="F27" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="13"/>
+      <c r="G27" s="29" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D28" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>11</v>
       </c>
       <c r="E28" s="7" t="s">
@@ -1510,115 +1684,123 @@
       <c r="F28" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G28" s="8"/>
+      <c r="G28" s="28" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C29" s="9" t="s">
+      <c r="A29" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G29" s="28" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G30" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F29" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G30" s="8"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="13"/>
+      <c r="D31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G31" s="29" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="E32" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" s="8"/>
+      <c r="E32" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="29" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>73</v>
+      <c r="A33" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G33" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -1626,10 +1808,10 @@
         <v>7</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>11</v>
@@ -1640,132 +1822,134 @@
       <c r="F34" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>76</v>
+      <c r="G34" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D35" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="13"/>
+      <c r="A35" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G35" s="29" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
-        <v>7</v>
+        <v>109</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D36" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G36" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E36" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="13" t="s">
-        <v>83</v>
+      <c r="F37" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>85</v>
+      <c r="A38" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>97</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="8" t="s">
-        <v>24</v>
+      <c r="E38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G38" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="D39" s="11" t="s">
+      <c r="A39" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E39" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>24</v>
+      <c r="E39" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G39" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D40" s="7" t="s">
         <v>11</v>
@@ -1776,91 +1960,91 @@
       <c r="F40" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G40" s="8" t="s">
-        <v>90</v>
+      <c r="G40" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="24" x14ac:dyDescent="0.35">
-      <c r="A42" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D42" s="6" t="s">
+      <c r="A41" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E42" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="8" t="s">
+      <c r="F41" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="s">
         <v>95</v>
+      </c>
+      <c r="B42" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G42" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="9" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="D43" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E43" s="12" t="s">
-        <v>11</v>
-      </c>
       <c r="F43" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G43" s="13" t="s">
-        <v>98</v>
+      <c r="G43" s="29" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
-        <v>87</v>
+        <v>7</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>11</v>
@@ -1868,22 +2052,20 @@
       <c r="F44" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G44" s="8" t="s">
-        <v>98</v>
-      </c>
+      <c r="G44" s="8"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>101</v>
+        <v>18</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>10</v>
+        <v>19</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E45" s="12" t="s">
         <v>11</v>
@@ -1891,22 +2073,20 @@
       <c r="F45" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G45" s="13" t="s">
-        <v>24</v>
-      </c>
+      <c r="G45" s="13"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>11</v>
       </c>
       <c r="E46" s="7" t="s">
         <v>11</v>
@@ -1914,63 +2094,59 @@
       <c r="F46" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G46" s="8" t="s">
-        <v>24</v>
-      </c>
+      <c r="G46" s="8"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="D47" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F47" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="13"/>
+      <c r="A47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G47" s="8"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D48" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="A48" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G48" s="13"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="9" t="s">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>108</v>
+        <v>34</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>109</v>
+        <v>35</v>
       </c>
       <c r="D49" s="12" t="s">
         <v>11</v>
@@ -1984,85 +2160,79 @@
       <c r="G49" s="13"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E50" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="24" x14ac:dyDescent="0.35">
-      <c r="A51" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="D51" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F51" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="13" t="s">
-        <v>114</v>
-      </c>
+      <c r="A50" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G50" s="13"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A51" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G51" s="8"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A52" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E52" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>118</v>
-      </c>
+      <c r="A52" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D52" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="13"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="9" t="s">
-        <v>115</v>
+        <v>7</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>119</v>
+        <v>61</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D53" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D53" s="22" t="s">
         <v>11</v>
       </c>
       <c r="E53" s="12" t="s">
@@ -2071,19 +2241,17 @@
       <c r="F53" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G53" s="13" t="s">
-        <v>120</v>
-      </c>
+      <c r="G53" s="13"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
-        <v>115</v>
+        <v>7</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>121</v>
+        <v>63</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>11</v>
@@ -2094,127 +2262,119 @@
       <c r="F54" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G54" s="8" t="s">
-        <v>122</v>
-      </c>
+      <c r="G54" s="8"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A55" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="D55" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F55" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G55" s="13" t="s">
-        <v>122</v>
-      </c>
+      <c r="A55" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G55" s="8"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F56" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="24" x14ac:dyDescent="0.35">
-      <c r="A57" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="B57" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C57" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F57" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G57" s="13" t="s">
-        <v>130</v>
-      </c>
+      <c r="A56" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F56" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" s="13"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A57" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G57" s="8"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G58" s="8" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="24" x14ac:dyDescent="0.35">
+      <c r="A58" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G58" s="13"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="9" t="s">
-        <v>133</v>
+        <v>95</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="D59" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E59" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G59" s="13" t="s">
-        <v>136</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G59" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G59" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G59" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G59">
+      <sortCondition ref="G1:G59"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -2231,7 +2391,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2242,16 +2402,16 @@
         <v>0</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -2273,7 +2433,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B5" s="16">
         <v>2</v>
@@ -2290,7 +2450,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B6" s="16">
         <v>5</v>
@@ -2307,7 +2467,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B7" s="16">
         <v>7</v>
@@ -2324,7 +2484,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="B8" s="16">
         <v>1</v>
@@ -2341,7 +2501,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="15" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="B9" s="16">
         <v>5</v>
@@ -2358,7 +2518,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="B10" s="17">
         <f>SUM(B4:B9)</f>
@@ -2379,7 +2539,7 @@
     </row>
     <row r="12" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>

</xml_diff>

<commit_message>
Ameliore la lisibilite du tableau de suivi des accords
- Colonnes resserrees + retour a la ligne (fin du texte coupe /
  des colonnes a 85 de large)
- Bordures fines, lignes alternees, categorie coloree (CCN, Accord
  local, NAO, DUE, Elections) pour reperer un type d'un coup d'oeil
- Cellules "manquant" surlignees en orange dans PDF/Word/Resume
- Filtres automatiques sur l'entete
- Feuille Synthese : bandeau de titre et tableau borde

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPDVVFk5WmrN62497A96pk
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -9,7 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi des accords" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthese" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Suivi des accords'!$A$1:$I$48</definedName>
+  </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +38,35 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="009C5700"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -49,8 +78,48 @@
         <fgColor rgb="FF14203A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0014203A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF1F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -58,16 +127,82 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,2096 +571,2097 @@
   <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="49.1796875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="84.81640625" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="17" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Thème</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Catégorie</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Date de signature</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>PDF signé</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Word d'origine</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Résumé</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Dépliant</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Nb dépliants</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Remarques</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Convention collective nationale des CLCC (texte intégral)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Consolidée au 1er juillet 2026</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>CCN des CLCC - 1er juillet 2026_.pdf</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Mise à jour au 1er juillet 2026 (était au 1er février 2026) : avenants 2026-01+01, 2026-05, 2026-06, avis A-9.1.6 intégrés par patch ciblé, vérifiés visuellement.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Télétravail</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>27/04/2021</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Accord Télétravail_signé.pdf</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Accord Télétravail_vdéfinitive.docx</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>resume-teletravail-2021.md</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Depliant_teletravail_FO.pdf</t>
         </is>
       </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="H3" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr"/>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Durée et aménagement du temps de travail — cadres</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>12/05/2021</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Cadres_signé.pdf</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Cadres_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>resume-att-cadres-2021.md</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Depliant_ATT_cadres_forfait_jours_FO.pdf · Depliant_ATT_cadres_en_heures_FO.pdf</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Avenant congés payés maladie (31/12/2025) désormais sur sa propre ligne, voir 'Avenant — Congés payés...'.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Avenant — Congés payés pendant un arrêt maladie (31/12/2025)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>Avenant ATT cadres incidences absences conges payes 2025.pdf</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Accord acquisition CP sur maladie - cadres.docx</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>resume-att-cadres-2021.md</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Depliant_ATT_cadres_forfait_jours_FO.pdf · Depliant_ATT_cadres_en_heures_FO.pdf</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ Signatures CGT-FO et Sud Santé-Sociaux manquantes (seuls DG et CFE-CGC ont signé). ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="120" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Durée et aménagement du temps de travail — non-cadres</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>14/09/2020 + avenant n°1 (heures sup) 31/01/2022</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Accord ATT Non Cadre + PV_Signé.pdf</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Non Cadre_VDéfinitive.docx</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>resume-att-non-cadres-2020.md</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Depliant_ATT_non_cadres_1_horaires_FO.pdf · Depliant_ATT_non_cadres_2_annualisation_FO.pdf · Depliant_ATT_non_cadres_3_conges_FO.pdf · Depliant_ATT_non_cadres_4_travail_de_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Avenant n°1 (heures sup, 2022) intégré au résumé. Avenant congés payés maladie (31/12/2025) désormais sur sa propre ligne, voir 'Avenant — Congés payés...'.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Avenant — Congés payés pendant un arrêt maladie (31/12/2025)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>31/12/2025</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Avenant ATT non cadres incidences absences conges payes 2025.pdf</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Accord acquisition CP sur maladie-Non cadres.docx</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>resume-att-non-cadres-2020.md</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Depliant_ATT_non_cadres_1_horaires_FO.pdf · Depliant_ATT_non_cadres_2_annualisation_FO.pdf · Depliant_ATT_non_cadres_3_conges_FO.pdf · Depliant_ATT_non_cadres_4_travail_de_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ ANOMALIE : signature du DG absente (CGT-FO, Sud Santé-Sociaux et CFE-CGC ont signé, pas l'employeur) — à clarifier avec la Direction. Ajouté quand même, signalé clairement (décision David 19/10/2026).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="105" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Compteur intermédiaire — personnel non posté</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>23/03/2024</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Avenant accord ATT_ Mise en place compteur intermédiaire_Salariés non postés.pdf</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire non postés version finale.docx</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>resume-compteur-intermediaire.md</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>Depliant_compteur_intermediaire_FO.pdf</t>
         </is>
       </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="H8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>Accord distinct de 'Compteur intermédiaire — personnel posté' (résumé/dépliant partagés). Séparé en 2 lignes le 19/10/2026 (1 ligne par accord). Signatures vérifiées : CGT-FO et CFE-CGC visibles, Sud Santé-Sociaux non visible.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Compteur intermédiaire — personnel posté</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>21/06/2024</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire salarié posté_signé.pdf</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire salarié posté_versiondéfinitive.docx</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>resume-compteur-intermediaire.md</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Depliant_compteur_intermediaire_FO.pdf</t>
         </is>
       </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="H9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Accord distinct de 'personnel non posté' (résumé/dépliant partagés). Nouvelle ligne le 19/10/2026 ; PDF et texte intégral désormais tous deux reliés.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Compte Épargne Temps (CET)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>2021 (base, PDF non retrouvé) + avenant 2022</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Accord CET_Avenant n1_signé.pdf</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>resume-cet-avenant-2022.md</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Depliant_CET_FO.pdf</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="H10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Fichier orphelin 'vDéfinitive' supprimé le 21/09/2026 (confirmé David) — accord de base 2021 toujours sans PDF ni Word.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>CDD à objet défini</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>Accord CDD à objet défini_Signé.pdf</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Accord CDD à objet défini_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>resume-cdd-objet-defini-2021.md</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Depliant_CDD_objet_defini_FO.pdf</t>
         </is>
       </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="H11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>PERCOL (épargne retraite collective)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Accord PERCOL_Signé.pdf</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>Accord PERCOL_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>resume-percol-2021.md</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Depliant_PERCOL_FO.pdf</t>
         </is>
       </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="H12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Congé humanitaire</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Accord Congé Humanitaire (2026).pdf</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Accord sur le congé humanitaire V2.docx</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>resume-conge-humanitaire-2026.md</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Depliant_conge_humanitaire_FO.pdf</t>
         </is>
       </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="H13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Égalité femmes-hommes</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>2026 (version en vigueur)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Accord égalité FH 2026.pdf</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Accord Egalité F H_V2026 05 20.docx</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>resume-egalite-fh-2026.md</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>Depliant_egalite_femmes_hommes_FO.pdf</t>
         </is>
       </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="H14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Travail de nuit</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>Accord travail de nuit - 2026.pdf</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Accord  nuit V 2026 05 04.docx</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>resume-travail-nuit-2026.md</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Depliant_stages_de_jour_personnel_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="H15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Validation des Acquis Professionnels (VAP)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>22/03/2024</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Accord sur la validation des acquis professionnels _Version signée.pdf</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Accord sur la validation des acquis professionnels V2025-2.docx</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>resume-vap-2025.md</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Depliant_VAP_FO.pdf</t>
         </is>
       </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="H16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Avenant du 04/02/2025 désormais sur sa propre ligne (voir 'Avenant — VAP').</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="75" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Avenant — VAP (04/02/2025)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>04/02/2025</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>Avenant à l'accord d'entreprise relatif à la Validation des Acquis Professionnels _04.02.2025_0.pdf</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>resume-vap-2025.md</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Depliant_VAP_FO.pdf</t>
         </is>
       </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="H17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Confirmé : porte l'étiquette V2025-2, cohérente avec le Word conservé.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Répartition de la BIC</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>2025 (V2025-2)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Accord relatif à la répartition de la BIC_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Accord sur la répartition de la BIC V2025-2.docx</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>resume-bic-2025.md</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>Depliant_BIC_FO.pdf</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>1</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="H18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Intéressement</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Accord d'entreprise relatif à l'intéressement (2026).pdf</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Accord  intéressement 2026 _ Version 4 (22.05.2026).docx</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>resume-interessement-2026.md</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Depliant_interessement_FO.pdf</t>
         </is>
       </c>
-      <c r="H19" t="n">
-        <v>1</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="H19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="75" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Forfait Mobilité Durable</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>24/10/2025</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Accord Forfait Mobilite Durable 2025.pdf</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Accord Forfait Mobilité Durable Vfinale.docx</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>resume-forfait-mobilite-durable-2025.md</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Depliant_forfait_mobilite_durable_FO.pdf</t>
         </is>
       </c>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="H20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant) : daté du 24/10/2025, signé DG/CGT-FO/CFE-CGC. ⚠️ Sud Santé-Sociaux n'a pas signé (ligne vide).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Prime chaussures</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>21/06/2023</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Accord prime chaussure version signée.pdf</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>Accord Prime Chaussures V finale.docx</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>resume-prime-chaussures-2023.md</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>Depliant_prime_chaussures_FO.pdf</t>
         </is>
       </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="H21" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Prime USC</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Accord prime USC signé.pdf</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Accord prime USC V finale.docx</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>resume-prime-usc-2023.md</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>Depliant_prime_USC_FO.pdf</t>
         </is>
       </c>
-      <c r="H22" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="H22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>Avenant du 26/04/2024 désormais sur sa propre ligne (voir 'Avenant — Prime USC').</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Avenant — Prime USC (26/04/2024)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>26/04/2024</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>AVENANT ACCORD PRIME USC_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>resume-prime-usc-2023.md</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Depliant_prime_USC_FO.pdf</t>
         </is>
       </c>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="H23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Aucun Word reçu.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>PVA</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Accord PVA_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Accord PVA_vFinale.docx</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>resume-pva-2022.md</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>Depliant_PVA_FO.pdf</t>
         </is>
       </c>
-      <c r="H24" t="n">
-        <v>1</v>
-      </c>
-      <c r="I24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="H24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Prime de retour inopiné (DUE, non négociée)</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>01/05/2024 (DUE, non négociée)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>DUE_Prime de retour inopiné.pdf</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>DUE_Prime de retour inopiné 01.05.2024 _ MER IDE AS.docx</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>resume-prime-retour-inopine.md</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_retour_inopine_FO.pdf</t>
         </is>
       </c>
-      <c r="H25" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="H25" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Parcours professionnel — Assistants Médicaux</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Accord relatif au parcours des assistantes médicales_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Accord parcours AM Version finale.docx</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>resume-parcours-am-2025.md</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Depliant_parcours_assistant_medical_FO.pdf</t>
         </is>
       </c>
-      <c r="H26" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="H26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Parcours professionnel — IDE / MER</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>13/03/2025</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>Accord parcours IDE et MER_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>Accord parcours IDE et MER V 2025 03 13 - VF.docx</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>resume-parcours-ide-mer-2025.md</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>Depliant_parcours_IDE_MER_FO.pdf</t>
         </is>
       </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="H27" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Parcours professionnel — Physiciens médicaux</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Accord Parcours Phycisiens_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>Accord Physiciens médicaux 2022_vFinale.docx</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>resume-parcours-physiciens-2022.md</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Depliant_parcours_physiciens_medicaux_FO.pdf</t>
         </is>
       </c>
-      <c r="H28" t="n">
-        <v>1</v>
-      </c>
-      <c r="I28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="H28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Reprise d'ancienneté — MER / AS / IDE</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>Accord Reprise Expérience professionnelle MER-AS-IDE_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>Accord reprise ancienneté MER IDE AS_vFinale.docx</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>resume-reprise-anciennete-mer-as-ide-2022.md</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Depliant_reprise_anciennete_MER_IDE_AS_FO.pdf</t>
         </is>
       </c>
-      <c r="H29" t="n">
-        <v>1</v>
-      </c>
-      <c r="I29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="H29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30" ht="75" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Dialogue social</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Élections</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Accord dialogue social 2026.pdf</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Accord sur le dialogue social 2026_Version 03.docx</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>resume-dialogue-social-2026.md</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H30" t="n">
+      <c r="H30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="31" ht="75" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Vote électronique</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Élections</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>09/04/2026</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>ACCORD VOTE ELECTRONIQUE _ Elections professionnelles 2026.pdf</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Accord Vote électronique_v2026 04 09.docx</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>resume-vote-electronique-2026.md</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H31" t="n">
+      <c r="H31" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>DUE : parcours techniciens de laboratoire / macroscopie</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>DUE, non datée précisément</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>DUE Parcours techs de laboratoire-macroscopie_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>DUE Tech de labo d'anapath.docx</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>resume-due-parcours-macroscopie.md</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>Depliant_DUE_parcours_macroscopie_FO.pdf</t>
         </is>
       </c>
-      <c r="H32" t="n">
-        <v>1</v>
-      </c>
-      <c r="I32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="H32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="105" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>DUE : complémentaire frais de santé</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>19/06/2024 (DUE)</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>DUE regime frais de sante 2024.pdf</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>DUE CFS_v2024 05 27.docx</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>resume-due-complementaire-frais-sante.md</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>Depliant_DUE_complementaire_frais_sante_FO.pdf</t>
         </is>
       </c>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="H33" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : PDF signé retrouvé le 19/10/2026 (était manquant) — date réelle de signature 19/06/2024, PAS 27/05/2024 comme précédemment indiqué (27/05 était la date du Word, pas de la signature).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>DUE : prime pool remplacement — Assistantes Médicales</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>22/04/2024 (DUE)</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>DUE prime pool remplacement assistantes medicales 2024.pdf</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>DUE_Prime de Pool de remplacement _ Assistantes Médicales Vfinale.docx</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>resume-due-prime-pool-remplacement-am.md</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_pool_remplacement_FO.pdf</t>
         </is>
       </c>
-      <c r="H34" t="n">
-        <v>1</v>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="H34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>DUE : prime pool remplacement — AS / IDE</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>22/04/2024 (DUE)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>DUE prime pool remplacement AS IDE 2024.pdf</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>DUE_Prime de Pool de remplacement _ soignants Version Définitive.docx</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>resume-due-prime-pool-remplacement-soignants.md</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_pool_remplacement_FO.pdf</t>
         </is>
       </c>
-      <c r="H35" t="n">
-        <v>1</v>
-      </c>
-      <c r="I35" t="inlineStr">
+      <c r="H35" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="36" ht="45" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Chèques syndicaux</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>03/10/2022</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Accord-Chèques syndicaux_v signée.pdf</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>Accord chèques syndicaux_v2022-09-22.docx</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>resume-cheques-syndicaux.md</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>Depliant_cheques_syndicaux_FO.pdf</t>
         </is>
       </c>
-      <c r="H36" t="n">
-        <v>1</v>
-      </c>
-      <c r="I36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="H36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="45" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2023</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>08/06/2023</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>PV Desaccord NAO 2023.pdf</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>PV Desaccord NAO 2023.md</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H37" t="n">
+      <c r="H37" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="I37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2024</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>18/04/2024</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr">
         <is>
           <t>NAO 2024 - PV Désaccord.pdf</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>NAO 2024 - PV Desaccord.md</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H38" t="n">
+      <c r="H38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2025</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>13/10/2025</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>NAO 2025 - Procès verbal de désaccord.pdf</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>pv-desaccord-nao-2025.md</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="I39" s="8" t="inlineStr"/>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2026</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>NAO 2026 _PV de désaccord signé.pdf</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr">
         <is>
           <t>NAO 2026 _PV de desaccord signe.md</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Grille de rémunération et de classification — personnel non praticien</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="10" t="inlineStr">
         <is>
           <t>2025-01-01 (date tirée du nom du fichier)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>2025-01-01 Grille de rémunération CLCC non praticiens.pdf</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="8" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — corrigée à la date figurant dans le nom du fichier (2025-01-01), à confirmer.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="42" ht="105" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Grille de rémunération — praticiens</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>non précisée dans le fichier</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>Grille rémunération praticien.pdf</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H42" t="n">
+      <c r="H42" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="4" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — aucune date vérifiée dans le fichier lui-même, laissée non précisée plutôt que d'en inventer une.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="43" ht="75" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>Accord intergénérationnel</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
         <is>
           <t>30/01/2020</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>Accord Intergénérationnel du 30 01 2020_signé.pdf</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
         <is>
           <t>resume-intergenerationnel.md</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="8" t="inlineStr">
         <is>
           <t>Depliant_intergenerationnel_FO.pdf</t>
         </is>
       </c>
-      <c r="H43" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" t="inlineStr">
+      <c r="H43" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="8" t="inlineStr">
         <is>
           <t>Avenant du 15/09/2023 désormais sur sa propre ligne (voir 'Avenant — Accord intergénérationnel'). Avenant 2021 non en vigueur, archivé.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="44" ht="75" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Avenant — Accord intergénérationnel (15/09/2023)</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>15/09/2023</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>Avenant accord d'entreprise intergénérationnel_2023_Version signée.pdf</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>resume-intergenerationnel.md</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="4" t="inlineStr">
         <is>
           <t>Depliant_intergenerationnel_FO.pdf</t>
         </is>
       </c>
-      <c r="H44" t="n">
-        <v>1</v>
-      </c>
-      <c r="I44" t="inlineStr">
+      <c r="H44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Modifie l'art. 3.4.2 (temps partiel fin de carrière). Aucun Word reçu.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="45" ht="105" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>Plan d'Épargne d'Entreprise (PEE)</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>22/02/2019</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="8" t="inlineStr">
         <is>
           <t>Accord PEE signe par FO et CGC.pdf</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H45" t="n">
+      <c r="H45" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="8" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG le 22/02/2019 — CGT-FO et CFE-CGC signataires, CGT et Sud Santé-Sociaux non signataires. Pas encore de résumé/dépliant salarié.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="46" ht="105" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Avenant — Indemnité de restauration</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>15/11/2016</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Avenant indemnite restauration 2016.pdf</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H46" t="n">
+      <c r="H46" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Avenant n°1 à l'accord du 19/12/2013 (accord de base non retrouvé). Signé par le DG et les 4 OS. Pas encore de résumé/dépliant salarié.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="47" ht="105" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
         <is>
           <t>Don de jours de repos non pris</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
         <is>
           <t>09/01/2015</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>Accord don de jours de repos 2015.pdf</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="8" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG et les 4 OS. En-tête du PDF porte une date de projet non mise à jour (sans incidence). Pas encore de résumé/dépliant salarié.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="48" ht="120" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Charte unilatérale sur le droit à la déconnexion</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="11" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>22/06/2018 (DUE)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Charte deconnexion 2018.pdf</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H48" t="n">
+      <c r="H48" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). DUE (pas un accord négocié) : seule la CFE-CGC avait signé l'accord proposé, négociation non aboutie. Signée par le DG seul. Pas encore de résumé/dépliant salarié.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2539,105 +2675,109 @@
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Synthèse au 19 octobre 2026</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Documents suivis</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="16" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>PDF signés présents</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="18" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>PDF signés manquants</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Word d'origine manquants</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="18" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Résumés rédigés</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="16" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Documents sans résumé</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="18" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Dépliants produits</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="16" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Documents sans dépliant</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="18" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>Note : « Documents sans dépliant » comprend les exclusions volontaires (NAO, PV de désaccord, CCN et ses 2 grilles) et les 4 accords ajoutés le 19/10/2026 encore sans résumé/dépliant salarié (PEE, avenant indemnité de restauration, don de jours de repos, charte déconnexion). « Dialogue social » et « Vote électronique » sont retirés du catalogue/site depuis le 19/10/2026 mais restent suivis ici (documents sources conservés).</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:B12"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Precise l'absence de Word pour la CCN et ses grilles
La CCN et ses 2 grilles de remuneration sont des textes de branche
publies par la FNCLCC/Unicancer, jamais rediges localement par l'ICO :
aucun Word d'origine n'existera jamais pour ces 3 documents.

- catalogue.json : note ajoutee sur ccn-clcc, ccn-grille-non-praticiens
  et ccn-grille-praticiens
- Tableau de suivi : ces 3 lignes passent de "manquant" a
  "non applicable" en colonne Word d'origine (plus de surlignage
  orange, qui ne concerne que les vraies lacunes)
- Synthese : "Word d'origine manquants" 16 -> 13, nouvelle ligne
  "Word non applicable (textes de branche)" = 3

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPDVVFk5WmrN62497A96pk
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,8 +65,14 @@
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +124,11 @@
         <fgColor rgb="00EEF1F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -145,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -202,6 +213,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -629,7 +649,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Convention collective nationale des CLCC (texte intégral)</t>
@@ -650,9 +670,9 @@
           <t>CCN des CLCC - 1er juillet 2026_.pdf</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>manquant</t>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
@@ -670,7 +690,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Mise à jour au 1er juillet 2026 (était au 1er février 2026) : avenants 2026-01+01, 2026-05, 2026-06, avis A-9.1.6 intégrés par patch ciblé, vérifiés visuellement.</t>
+          <t>Mise à jour au 1er juillet 2026 (était au 1er février 2026) : avenants 2026-01+01, 2026-05, 2026-06, avis A-9.1.6 intégrés par patch ciblé, vérifiés visuellement. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2320,7 @@
       </c>
       <c r="I40" s="4" t="inlineStr"/>
     </row>
-    <row r="41" ht="90" customHeight="1">
+    <row r="41" ht="135" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Grille de rémunération et de classification — personnel non praticien</t>
@@ -2321,9 +2341,9 @@
           <t>2025-01-01 Grille de rémunération CLCC non praticiens.pdf</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>manquant</t>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -2341,11 +2361,11 @@
       </c>
       <c r="I41" s="8" t="inlineStr">
         <is>
-          <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — corrigée à la date figurant dans le nom du fichier (2025-01-01), à confirmer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="105" customHeight="1">
+          <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — corrigée à la date figurant dans le nom du fichier (2025-01-01), à confirmer. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="135" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Grille de rémunération — praticiens</t>
@@ -2366,9 +2386,9 @@
           <t>Grille rémunération praticien.pdf</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>manquant</t>
+      <c r="E42" s="21" t="inlineStr">
+        <is>
+          <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
@@ -2386,7 +2406,7 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — aucune date vérifiée dans le fichier lui-même, laissée non précisée plutôt que d'en inventer une.</t>
+          <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — aucune date vérifiée dans le fichier lui-même, laissée non précisée plutôt que d'en inventer une. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2724,51 +2744,64 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Résumés rédigés</t>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Word non applicable (textes de branche)</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Documents sans résumé</t>
+          <t>Résumés rédigés</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Dépliants produits</t>
+          <t>Documents sans résumé</t>
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>34</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
+          <t>Dépliants produits</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
           <t>Documents sans dépliant</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B11" s="16" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="12" ht="95" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Note : « Documents sans dépliant » comprend les exclusions volontaires (NAO, PV de désaccord, CCN et ses 2 grilles) et les 4 accords ajoutés le 19/10/2026 encore sans résumé/dépliant salarié (PEE, avenant indemnité de restauration, don de jours de repos, charte déconnexion). « Dialogue social » et « Vote électronique » sont retirés du catalogue/site depuis le 19/10/2026 mais restent suivis ici (documents sources conservés).</t>
         </is>
@@ -2776,7 +2809,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajoute les PV de desaccord NAO 2024 et 2025 au format Word d'origine
Fichiers Word verifies identiques au contenu du .md issu du PDF signe.
Signature verifiee visuellement sur le PDF : Pr Mario Campone (DG) seul
signataire sur les deux PV, coherent avec leur nature de PV de desaccord
unilateral (18/04/2024 et 13/10/2025).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -2565,7 +2565,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>PV NAO 2024 - V Finale plus en vigueur.docx</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -2581,7 +2581,11 @@
       <c r="H38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Fichier Word ajouté le 20/10/2026 par David Di Peri. Contenu comparé intégralement au .md existant (lui-même issu du PDF signé) : aucun écart trouvé. Date et signature (Pr Mario Campone, Directeur Général, seul signataire) verifiees visuellement sur le PDF signe le 20/10/2026 : conformes (18/04/2024).</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
@@ -2606,7 +2610,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>PV NAO 2025 - V 2 plus en vigueur.docx</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -2622,7 +2626,11 @@
       <c r="H39" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="8" t="inlineStr"/>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Fichier Word ajouté le 20/10/2026 par David Di Peri. Contenu comparé intégralement au .md existant (lui-même issu du PDF signé) : aucun écart trouvé. Date et signature (Pr Mario Campone, Directeur Général, seul signataire) verifiees visuellement sur le PDF signe le 20/10/2026 : conformes (13/10/2025).</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="A40" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Ajoute le PDF signe de l'accord CET de base (19/03/2021), retrouve chez David
Le PDF de l'accord de base manquait (seul l'avenant n1 de 2022 en avait un) ;
le .md existait a partir d'un Word de travail, jamais verifie contre un PDF signe.

Verification visuelle du PDF (titre, preambule, articles 1 a 8, plafonds
1820h/35h/20j) : contenu du .md confirme fidele au texte signe.

Point a signaler : sur la page de signature, Sud Sante-Sociaux (Isabelle
Fouillet) n'a pas de signature visible, alors qu'elle est citee comme partie
a l'accord - meme constat que pour l'avenant n1 (2022). Resume et dependant
corriges en consequence (ne citent plus Sud Sante-Sociaux comme signataire).
Catalogue et tableau de suivi mis a jour.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -1098,12 +1098,12 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>2021 (base, PDF non retrouvé) + avenant 2022</t>
+          <t>19/03/2021 (base) + avenant 31/01/2022</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Accord CET_Avenant n1_signé.pdf</t>
+          <t>accord-cet-2021.pdf (base) + Accord CET_Avenant n1_signé.pdf (avenant)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Fichier orphelin 'vDéfinitive' supprimé le 21/09/2026 (confirmé David) — accord de base 2021 toujours sans PDF ni Word.</t>
+          <t>PDF de l'accord de base retrouve et integre le 20/10/2026 (David l'a ajoute dans son dossier local). Signatures verifiees visuellement sur le PDF de base (19/03/2021) : ICO (Campone), CGT-FO, CFDT, CFE-CGC ont signe ; Sud Sante-Sociaux (Isabelle Fouillet), partie a l'accord, n'a pas de signature visible sur la page de signature — meme constat que pour l'avenant n1 (31/01/2022), deja note ci-dessus. Contenu du .md verifie conforme au PDF signe (preambule, articles 1 a 8, plafonds).</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">

</xml_diff>

<commit_message>
Met a jour la navigation, le catalogue et le tableau de suivi pour la rubrique Prevoyance
Ajoute la rubrique dans mkdocs.yml, les nouvelles entrees dans le catalogue du site, les lignes du tableau de suivi (avec la coquille de titre des DUE 2022 signalee) et un renvoi depuis l'index DUE.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Incoherence de date entre le corps (signee 'le 19 juin 2024') et le coupon-reponse (mentionne une decision 'datee du 1er juin 2024') -- confusion entre date de signature et date d'effet du regime. Art. 3 : les dispenses n5/6 (art. R.242-1-6) reprennent presque mot pour mot les dispenses n1/2 (L.911-7 III/D.911-2) sans que la difference pratique soit clairement expliquee.</t>
+          <t>Incoherence de date entre le corps (signee 'le 19 juin 2024') et le coupon-reponse (mentionne une decision 'datee du 1er juin 2024') -- confusion entre date de signature et date d'effet du regime. Art. 3 : les dispenses n5/6 (art. R.242-1-6) reprennent presque mot pour mot les dispenses n1/2 (L.911-7 III/D.911-2) sans que la difference pratique soit clairement expliquee. | Un regime anterieur (2022, scinde cadre/non cadre) portait par erreur le titre 'Prevoyance' alors qu'il s'agit du meme regime frais de sante -- voir dossier prevoyance-mutuelle-retraite.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3215,6 +3215,251 @@
       <c r="K51" t="inlineStr">
         <is>
           <t>Aucune clause de bilan, de révision périodique ou de commission de suivi identifiée dans le texte : la seule procédure de modification prévue (art. 4.2) est la reprise de la procédure légale complète (avis du CSE Central) en cas de changement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance (en realite frais de sante) 2022 - Non cadre</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>DUE</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>25/04/2022 (DUE)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance 2022 Non cadre ICO.pdf</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes).</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance (en realite frais de sante) 2022 - Cadre</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DUE</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>25/04/2022 (DUE)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance 2022 Cadre ICO.pdf</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Difference avec la version non cadre : perimetre (positions 6-7 CCN + praticiens) et cotisations (3 tranches PASS au lieu de 2, taux differents).</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Prevoyance AXA (deces, incapacite, invalidite) - Non cadre</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Notice prevoyance non cadres AXA 2015.pdf</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604120000Q. Garanties verifiees identiques mot pour mot a la version cadre (comparaison textuelle programmatique page par page) -- seul le perimetre des beneficiaires et le numero de contrat different. Resume unique cadre+non cadre avec clause beneficiaire integree.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Information individuelle (notice remise a chaque salarie, Art. 9) ; portabilite en cas de rupture ouvrant droit au chomage (maintien loi 2013) ; maintien des garanties deces au profit des beneficiaires de rentes en cas de changement d'organisme assureur (Art. 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Prevoyance AXA (deces, incapacite, invalidite) - Cadre</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Notice prevoyance cadres AXA 2015.pdf</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604110000Q. Garanties identiques a la version non cadre (voir ligne ci-dessus) -- meme resume et depliant, compte comme un seul depliant au total (Nb depliants=0 ici pour ne pas compter en double).</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Identique a la ligne non cadre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Clause beneficiaire Prevoyance AXA (formulaire)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>VF 2019</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Clause beneficiaire Prevoyance AXA 2019.pdf</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Integree dans resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Formulaire individuel AXA (reference 480299 04 2017), pas un document contractuel. Contenu integre a la section Clause beneficiaire du resume Prevoyance AXA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ICO Information Assistance AXA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ICO Information Assistance AXA.pdf</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Non (en attente de validation David)</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Assistances AXA : resume, depliant, rangement dans la rubrique Prevoyance
Corrige le .md source (condition 50 km limitee a la presence d'un proche, limite garde enfants).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -3451,15 +3451,20 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Non (en attente de validation David)</t>
+          <t>resume-assistance-axa.md (20/10/2026)</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Depliant_Assistances_AXA_FO.pdf (20/10/2026)</t>
         </is>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer.</t>
+          <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer. Resume redige et integre le 20/10/2026 sur demande de David : notice d'information des assistances AXA possibles. Erreur corrigee dans le .md source : la condition "aucun membre de la famille a moins de 50 km" ne vise que la presence d'un proche au chevet.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tableau de suivi : synthese recalculee, remarques sur les 7 PDF servis par le site
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -976,7 +976,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="165" customHeight="1">
+    <row r="7" ht="180" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Avenant — ATT non cadres : CET heures supplémentaires (31/01/2022)</t>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Ligne séparée le 20/10/2026 (était fondue dans la ligne de l'accord de base). Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). ⚠️ L'en-tête du .md liste les signataires sans l'ICO alors que la signature du DG figure sur le PDF. Mis à la signature du 31/01 au 11/02/2022 (art. 2.2). Transcription Markdown issue du Word, non comparée au PDF dans cette passe.</t>
+          <t>Ligne séparée le 20/10/2026 (était fondue dans la ligne de l'accord de base). Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). ⚠️ L'en-tête du .md liste les signataires sans l'ICO alors que la signature du DG figure sur le PDF. Mis à la signature du 31/01 au 11/02/2022 (art. 2.2). Transcription Markdown issue du Word, non comparée au PDF dans cette passe. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K7" s="25" t="inlineStr">
@@ -1276,7 +1276,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="135" customHeight="1">
+    <row r="12" ht="150" customHeight="1">
       <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Avenant — CET n°1 (31/01/2022)</t>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ligne séparée le 20/10/2026. Annule et remplace l'art. 3.3 (alimentation du CET) de l'accord du 19/03/2021 ; date limite de dépôt des éléments temporels fixée au 15 janvier. Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). Mis à la signature du 31/01 au 11/02/2022.</t>
+          <t>Ligne séparée le 20/10/2026. Annule et remplace l'art. 3.3 (alimentation du CET) de l'accord du 19/03/2021 ; date limite de dépôt des éléments temporels fixée au 15 janvier. Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). Mis à la signature du 31/01 au 11/02/2022. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K12" s="25" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé.</t>
+          <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K32" s="25" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé.</t>
+          <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K33" s="25" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>20/10/2026 : doublon avec accent supprimé (PDF « v signée »). Pas de dépliant (hors périmètre dépliant).</t>
+          <t>20/10/2026 : doublon avec accent supprimé (PDF « v signée »). Pas de dépliant (hors périmètre dépliant). PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K38" s="25" t="inlineStr">
@@ -3510,7 +3510,7 @@
       </c>
       <c r="J51" s="25" t="inlineStr">
         <is>
-          <t>Restaure le 20/10/2026 -- avait ete classe a tort 'plus en vigueur' et archive ; aucun texte posterieur ne l'abroge (regle avenants, David 20/10/2026). Ajoute la possibilite de fractionner un temps partiel a 50% sur 2 semaines (Art. 3.4.2).</t>
+          <t>Restaure le 20/10/2026 -- avait ete classe a tort 'plus en vigueur' et archive ; aucun texte posterieur ne l'abroge (regle avenants, David 20/10/2026). Ajoute la possibilite de fractionner un temps partiel a 50% sur 2 semaines (Art. 3.4.2). PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K51" s="25" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="J52" s="25" t="inlineStr">
         <is>
-          <t>Ligne ajoutee le 20/10/2026 (absente du tableau jusqu'ici). 20/10/2026 : PDF signé et Word retrouvés dans le dépôt (la ligne les indiquait manquants).</t>
+          <t>Ligne ajoutee le 20/10/2026 (absente du tableau jusqu'ici). 20/10/2026 : PDF signé et Word retrouvés dans le dépôt (la ligne les indiquait manquants). PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
       <c r="K52" s="25" t="inlineStr">
@@ -4022,7 +4022,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Synthèse mise à jour le 20 octobre 2026</t>
+          <t>Synthèse recalculée le 20 octobre 2026 (une ligne du tableau = un document)</t>
         </is>
       </c>
       <c r="B1" s="14" t="n"/>
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -4044,7 +4044,7 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
@@ -4064,17 +4064,17 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="23" t="inlineStr">
         <is>
-          <t>Word non applicable (textes de branche)</t>
+          <t>Word non applicable (branche + assureur)</t>
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -4084,7 +4084,7 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="B9" s="16" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="B10" s="18" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11">
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -4123,7 +4123,7 @@
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="20" t="inlineStr">
         <is>
-          <t>Note : mise à jour du 20/10/2026 : PEE, avenant indemnité de restauration, don de jours et charte déconnexion ont désormais un résumé et un dépliant (+4 résumés, +4 dépliants, -4 documents sans résumé, -4 sans dépliant par rapport au 19/10). « Documents sans dépliant » comprend les exclusions volontaires (NAO, PV de désaccord, CCN et ses 2 grilles). Chèques syndicaux : pas de dépliant (hors périmètre). ⚠️ Les lignes « PDF manquants » et « Word manquants » n'ont pas été recalculées : leur mode de calcul d'origine n'est pas documenté, à recompter avec David (le tableau détaillé fait foi). « Dialogue social » et « Vote électronique » sont retirés du catalogue/site depuis le 19/10/2026 mais restent suivis ici.</t>
+          <t>Note : chiffres recalculés le 20/10/2026 à partir des lignes du tableau (58 lignes dont 9 avenants). « Résumés rédigés » compte les lignes rattachées à un résumé (un avenant partage le résumé de son accord de base ; les 4 PV de désaccord NAO sont des transcriptions, pas des résumés). « Dépliants produits » compte les fichiers PDF (36), « Documents sans dépliant » les lignes sans dépliant (NAO, PV de désaccord, CCN et grilles, dialogue social, vote électronique, chèques syndicaux, documents assureur). Les 7 PDF servis par le site sans être listés ont leur lien sur le Thème.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tableau de suivi : avenants sous leurs accords, couleurs par categorie, bordures et mise en forme
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -11,6 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Suivi des accords'!$A$1:$L$59</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Suivi des accords'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +78,25 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -135,8 +153,41 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4DFEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F0EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -158,11 +209,53 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00A6A6A6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00A6A6A6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00A6A6A6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00A6A6A6"/>
+      </right>
+      <top style="medium">
+        <color rgb="00404040"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00404040"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -243,6 +336,279 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -607,3338 +973,3106 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="13" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
-    <col width="38" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Thème</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="89" t="inlineStr">
+        <is>
+          <t>Accord</t>
+        </is>
+      </c>
+      <c r="B1" s="89" t="inlineStr">
+        <is>
+          <t>Avenant</t>
+        </is>
+      </c>
+      <c r="C1" s="89" t="inlineStr">
         <is>
           <t>Catégorie</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Sous catégorie</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="89" t="inlineStr">
         <is>
           <t>Date de signature</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="89" t="inlineStr">
         <is>
           <t>PDF signé</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="89" t="inlineStr">
         <is>
           <t>Word d'origine</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="89" t="inlineStr">
         <is>
           <t>Résumé</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="89" t="inlineStr">
         <is>
           <t>Dépliant</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="89" t="inlineStr">
         <is>
           <t>Nb dépliants</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="89" t="inlineStr">
         <is>
           <t>Remarques</t>
         </is>
       </c>
-      <c r="K1" s="24" t="inlineStr">
+      <c r="K1" s="90" t="inlineStr">
         <is>
           <t>Coquilles relevees (20/10/2026)</t>
         </is>
       </c>
-      <c r="L1" s="24" t="inlineStr">
+      <c r="L1" s="90" t="inlineStr">
         <is>
           <t>Moyens de controle / clauses de suivi (20/10/2026)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="90" customHeight="1">
-      <c r="A2" s="26" t="inlineStr">
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t>Convention collective nationale des CLCC (texte intégral)</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="92" t="n"/>
+      <c r="C2" s="93" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="93" t="inlineStr">
         <is>
           <t>Consolidée au 1er juillet 2026</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="94" t="inlineStr">
         <is>
           <t>CCN des CLCC - 1er juillet 2026_.pdf</t>
         </is>
       </c>
-      <c r="F2" s="21" t="inlineStr">
+      <c r="F2" s="94" t="inlineStr">
         <is>
           <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="94" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I2" s="6" t="n">
+      <c r="I2" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="94" t="inlineStr">
         <is>
           <t>Mise à jour au 1er juillet 2026 (était au 1er février 2026) : avenants 2026-01+01, 2026-05, 2026-06, avis A-9.1.6 intégrés par patch ciblé, vérifiés visuellement. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
         </is>
       </c>
-      <c r="K2" s="25" t="n"/>
-      <c r="L2" s="25" t="n"/>
-    </row>
-    <row r="3" ht="120" customHeight="1">
-      <c r="A3" s="27" t="inlineStr">
+      <c r="K2" s="94" t="n"/>
+      <c r="L2" s="94" t="n"/>
+    </row>
+    <row r="3" ht="87" customHeight="1">
+      <c r="A3" s="95" t="inlineStr">
         <is>
           <t>Télétravail</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="92" t="n"/>
+      <c r="C3" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
+      <c r="D3" s="96" t="inlineStr">
         <is>
           <t>27/04/2021</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="97" t="inlineStr">
         <is>
           <t>Accord Télétravail_signé.pdf</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="97" t="inlineStr">
         <is>
           <t>Accord Télétravail_vdéfinitive.docx</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="97" t="inlineStr">
         <is>
           <t>resume-teletravail-2021.md</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="97" t="inlineStr">
         <is>
           <t>Depliant_teletravail_FO.pdf</t>
         </is>
       </c>
-      <c r="I3" s="10" t="n">
+      <c r="I3" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="25" t="inlineStr">
+      <c r="J3" s="97" t="n"/>
+      <c r="K3" s="97" t="inlineStr">
         <is>
           <t>Saut de numerotation : Art. 5.1 'Clause de reversibilite' puis directement Art. 5.3 'Suspension du teletravail' -- le 5.2 est manquant. Renvoi incoherent (~art. 4.3) vers 'l'article 5.1' pour une periode d'adaptation qui n'y est pas traitee. Faute : 'execution' orthographie 'execution' (6 mois d'anciennete).</t>
         </is>
       </c>
-      <c r="L3" s="25" t="inlineStr">
+      <c r="L3" s="97" t="inlineStr">
         <is>
           <t>Commission de suivi CSSCT centrale &gt;=1x/an (missions detaillees), rubrique bilan social, saisine ad hoc, clause de revoyure a 1 an (Art. 12.1) ; duree indeterminee (12.2) ; revision (12.3) ; denonciation (12.4).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="135" customHeight="1">
-      <c r="A4" s="26" t="inlineStr">
+    <row r="4" ht="87" customHeight="1">
+      <c r="A4" s="95" t="inlineStr">
         <is>
           <t>Durée et aménagement du temps de travail — cadres</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="97" t="n"/>
+      <c r="C4" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="96" t="inlineStr">
         <is>
           <t>12/05/2021</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="97" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Cadres_signé.pdf</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="97" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Cadres_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="97" t="inlineStr">
         <is>
           <t>resume-att-cadres-2021.md</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="97" t="inlineStr">
         <is>
           <t>Depliant_ATT_cadres_forfait_jours_FO.pdf · Depliant_ATT_cadres_en_heures_FO.pdf</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n">
+      <c r="I4" s="96" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="97" t="inlineStr">
         <is>
           <t>Avenant congés payés maladie (31/12/2025) désormais sur sa propre ligne, voir 'Avenant — Congés payés...'.</t>
         </is>
       </c>
-      <c r="K4" s="25" t="inlineStr">
+      <c r="K4" s="97" t="inlineStr">
         <is>
           <t>Numerotation incoherente : la section '1.3 Garanties' contient des sous-articles numerotes 1.1.1 a 1.1.5 au lieu de 1.3.1-1.3.5 (dispositif d'alerte charge de travail = 1.1.4, entretien annuel = 1.1.5). Art. 2.1 'Cadres concernes' renvoie a tort a 'l'article 2.1' pour le forfait jours autonome (en realite defini a l'Article 1).</t>
         </is>
       </c>
-      <c r="L4" s="25" t="inlineStr">
+      <c r="L4" s="97" t="inlineStr">
         <is>
           <t>Commission de suivi (delegues syndicaux, Art. 4.1) ; bilan quantitatif/qualitatif (4.1) ; suivi individuel forfait jours -- document de controle mensuel, dispositif d'alerte, entretien annuel (Art. 1.3, numerote a tort 1.1.3-1.1.5) ; duree indeterminee (4.2) ; revision (4.3) ; denonciation (4.4).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="180" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+    <row r="5" ht="127.5" customHeight="1">
+      <c r="A5" s="98" t="n"/>
+      <c r="B5" s="99" t="inlineStr">
         <is>
           <t>Avenant — Congés payés pendant un arrêt maladie (31/12/2025)</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="C5" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="100" t="inlineStr">
         <is>
           <t>31/12/2025</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="98" t="inlineStr">
         <is>
           <t>Avenant ATT cadres incidences absences conges payes 2025.pdf</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="98" t="inlineStr">
         <is>
           <t>Accord acquisition CP sur maladie - cadres.docx</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G5" s="98" t="inlineStr">
         <is>
           <t>resume-att-cadres-2021.md</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="98" t="inlineStr">
         <is>
           <t>Depliant_ATT_cadres_forfait_jours_FO.pdf · Depliant_ATT_cadres_en_heures_FO.pdf</t>
         </is>
       </c>
-      <c r="I5" s="10" t="n">
+      <c r="I5" s="100" t="n">
         <v>2</v>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="J5" s="98" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ Signatures CGT-FO et Sud Santé-Sociaux manquantes (seuls DG et CFE-CGC ont signé). ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.</t>
         </is>
       </c>
-      <c r="K5" s="25" t="inlineStr">
+      <c r="K5" s="98" t="inlineStr">
         <is>
           <t>Le texte evoque par erreur 'l'amenagement du temps de travail des salaries non-cadre' alors que cet avenant concerne les CADRES (deja signale dans le resume). 'remplacer ... et annuelle' au lieu de 'annule' (faute). Numerotation '4.4 Formalites de depot' alors que la section est '2.1-2.3' (Article 2 -- Dispositions finales) : devrait etre 2.4. Sur le PDF signe, seuls le DG et la CFE-CGC ont signe (CGT-FO et Sud Sante-Sociaux non signataires).</t>
         </is>
       </c>
-      <c r="L5" s="25" t="inlineStr">
+      <c r="L5" s="98" t="inlineStr">
         <is>
           <t>Mecanismes propres a l'avenant (Art. 2.1-2.3) : revision, duree, denonciation -- repris dans la section Suivi du resume ATT cadres.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+    <row r="6" ht="114" customHeight="1">
+      <c r="A6" s="95" t="inlineStr">
         <is>
           <t>Durée et aménagement du temps de travail — non-cadres</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="97" t="n"/>
+      <c r="C6" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="96" t="inlineStr">
         <is>
           <t>14/09/2020</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="97" t="inlineStr">
         <is>
           <t>Accord ATT Non Cadre + PV_Signé.pdf</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="97" t="inlineStr">
         <is>
           <t>Accord Durée et ATT Non Cadre_VDéfinitive.docx</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="97" t="inlineStr">
         <is>
           <t>resume-att-non-cadres-2020.md</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="97" t="inlineStr">
         <is>
           <t>Depliant_ATT_non_cadres_1_horaires_FO.pdf · Depliant_ATT_non_cadres_2_annualisation_FO.pdf · Depliant_ATT_non_cadres_3_conges_FO.pdf · Depliant_ATT_non_cadres_4_travail_de_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="96" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="97" t="inlineStr">
         <is>
           <t>Avenant n°1 (CET heures supplémentaires, 31/01/2022) et avenant congés payés maladie (31/12/2025) : voir leurs lignes dédiées (séparées le 20/10/2026). Les deux sont intégrés au résumé.</t>
         </is>
       </c>
-      <c r="K6" s="25" t="inlineStr">
+      <c r="K6" s="97" t="inlineStr">
         <is>
           <t>Aucune coquille dans le corps de l'accord 2020 lui-meme (numerotation 1.x-5.x coherente).</t>
         </is>
       </c>
-      <c r="L6" s="25" t="inlineStr">
+      <c r="L6" s="97" t="inlineStr">
         <is>
           <t>Commission de suivi (delegues syndicaux, Art. 5.1) ; bilan quantitatif/qualitatif (5.1) ; duree indeterminee/entree en vigueur (5.2) ; revision (5.3) ; denonciation (5.4).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="180" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+    <row r="7" ht="114" customHeight="1">
+      <c r="A7" s="98" t="n"/>
+      <c r="B7" s="99" t="inlineStr">
         <is>
           <t>Avenant — ATT non cadres : CET heures supplémentaires (31/01/2022)</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="C7" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="100" t="inlineStr">
         <is>
           <t>31/01/2022</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="98" t="inlineStr">
         <is>
           <t>Accord ATT NC_Avenant n1_Signé.pdf</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="98" t="inlineStr">
         <is>
           <t>Accord ATT NC_Avenant n°1_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="98" t="inlineStr">
         <is>
           <t>resume-att-non-cadres-2020.md</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="98" t="inlineStr">
         <is>
           <t>Depliant_ATT_non_cadres_1_horaires_FO.pdf · Depliant_ATT_non_cadres_2_annualisation_FO.pdf</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="100" t="n">
         <v>2</v>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="98" t="inlineStr">
         <is>
           <t>Ligne séparée le 20/10/2026 (était fondue dans la ligne de l'accord de base). Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). ⚠️ L'en-tête du .md liste les signataires sans l'ICO alors que la signature du DG figure sur le PDF. Mis à la signature du 31/01 au 11/02/2022 (art. 2.2). Transcription Markdown issue du Word, non comparée au PDF dans cette passe. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
-      <c r="K7" s="25" t="inlineStr">
+      <c r="K7" s="98" t="inlineStr">
         <is>
           <t>Aucune coquille relevée dans cette passe.</t>
         </is>
       </c>
-      <c r="L7" s="25" t="inlineStr">
+      <c r="L7" s="98" t="inlineStr">
         <is>
           <t>Durée indéterminée ; entrée en vigueur le lendemain du dépôt (art. 2.1). Pas de commission de suivi propre à l'avenant.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="150" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
+    <row r="8" ht="114" customHeight="1">
+      <c r="A8" s="98" t="n"/>
+      <c r="B8" s="99" t="inlineStr">
         <is>
           <t>Avenant — Congés payés pendant un arrêt maladie (31/12/2025)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="C8" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="100" t="inlineStr">
         <is>
           <t>31/12/2025</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="98" t="inlineStr">
         <is>
           <t>Avenant ATT non cadres incidences absences conges payes 2025.pdf</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="98" t="inlineStr">
         <is>
           <t>Accord acquisition CP sur maladie-Non cadres.docx</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="98" t="inlineStr">
         <is>
           <t>resume-att-non-cadres-2020.md</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="98" t="inlineStr">
         <is>
           <t>Depliant_ATT_non_cadres_1_horaires_FO.pdf · Depliant_ATT_non_cadres_2_annualisation_FO.pdf · Depliant_ATT_non_cadres_3_conges_FO.pdf · Depliant_ATT_non_cadres_4_travail_de_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="I8" s="10" t="n">
+      <c r="I8" s="100" t="n">
         <v>4</v>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="J8" s="98" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ ANOMALIE : signature du DG absente (CGT-FO, Sud Santé-Sociaux et CFE-CGC ont signé, pas l'employeur) — à clarifier avec la Direction. Ajouté quand même, signalé clairement (décision David 19/10/2026).</t>
         </is>
       </c>
-      <c r="K8" s="25" t="inlineStr">
+      <c r="K8" s="98" t="inlineStr">
         <is>
           <t>'les devenir' (accord fautif, devrait etre 'le devenir') ; 'remplace et annuelle' au lieu de 'annule' (meme faute que la version cadres) ; numerotation '4.4 Formalites de depot' alors que la section est 'Article 2' (devrait etre 2.4). Sur le PDF signe, CGT-FO, Sud Sante-Sociaux et CFE-CGC ont signe mais PAS le Directeur General (deja signale dans le resume).</t>
         </is>
       </c>
-      <c r="L8" s="25" t="inlineStr">
+      <c r="L8" s="98" t="inlineStr">
         <is>
           <t>Mecanismes propres a l'avenant CET 2022 (Art. 2.1) et a l'avenant maladie 2025 (Art. 2.1-2.3) -- repris dans la section Suivi du resume ATT non-cadres.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="210" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
+    <row r="9" ht="141" customHeight="1">
+      <c r="A9" s="95" t="inlineStr">
         <is>
           <t>Compteur intermédiaire — personnel non posté</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="92" t="n"/>
+      <c r="C9" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="96" t="inlineStr">
         <is>
           <t>23/03/2024</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="97" t="inlineStr">
         <is>
           <t>Avenant accord ATT_ Mise en place compteur intermédiaire_Salariés non postés.pdf</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="97" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire non postés version finale.docx</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="97" t="inlineStr">
         <is>
           <t>resume-compteur-intermediaire.md</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="97" t="inlineStr">
         <is>
           <t>Depliant_compteur_intermediaire_FO.pdf</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I9" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="97" t="inlineStr">
         <is>
           <t>Accord distinct de 'Compteur intermédiaire — personnel posté' (résumé/dépliant partagés). Séparé en 2 lignes le 19/10/2026 (1 ligne par accord). Signatures vérifiées : CGT-FO et CFE-CGC visibles, Sud Santé-Sociaux non visible.</t>
         </is>
       </c>
-      <c r="K9" s="25" t="inlineStr">
+      <c r="K9" s="97" t="inlineStr">
         <is>
           <t>'bornes fixes' repete par erreur a deux endroits du paragraphe recuperation jusqu'a 1h (probablement 'bornes variables' pour l'autonomie, incoherent avec le Preambule qui distingue plages fixes/variables). Dates de signature incoherentes a l'Art. 4.4 ('18/3/2024au 2/3/2024', espace manquant, fin anterieure au debut). Art. 4.3 : 'DIRECCTE d'Angers' -- anachronisme (DREETS depuis avril 2021, accord signe en 2024). Corrige dans le resume : la regle 'des la 1ere minute' avait ete recopiee a tort du regime poste, qui ne la prevoit pas pour le non poste.</t>
         </is>
       </c>
-      <c r="L9" s="25" t="inlineStr">
+      <c r="L9" s="97" t="inlineStr">
         <is>
           <t>Revision (Art. 4.2) ; duree indeterminee et denonciation liee aux mandats CSE (4.1 et 4.3). Aucune commission de suivi ni bilan annuel identifie.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="95" t="inlineStr">
         <is>
           <t>Compteur intermédiaire — personnel posté</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="92" t="n"/>
+      <c r="C10" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D10" s="96" t="inlineStr">
         <is>
           <t>21/06/2024</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="97" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire salarié posté_signé.pdf</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="97" t="inlineStr">
         <is>
           <t>Accord compteur intermédiaire salarié posté_versiondéfinitive.docx</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="97" t="inlineStr">
         <is>
           <t>resume-compteur-intermediaire.md</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="H10" s="97" t="inlineStr">
         <is>
           <t>Depliant_compteur_intermediaire_FO.pdf</t>
         </is>
       </c>
-      <c r="I10" s="10" t="n">
+      <c r="I10" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J10" s="97" t="inlineStr">
         <is>
           <t>Accord distinct de 'personnel non posté' (résumé/dépliant partagés). Nouvelle ligne le 19/10/2026 ; PDF et texte intégral désormais tous deux reliés.</t>
         </is>
       </c>
-      <c r="K10" s="25" t="inlineStr">
+      <c r="K10" s="97" t="inlineStr">
         <is>
           <t>Aucune coquille supplementaire relevee (texte coherent, terminologie DREETS correcte pour sa date de signature 21/06/2024).</t>
         </is>
       </c>
-      <c r="L10" s="25" t="inlineStr">
+      <c r="L10" s="97" t="inlineStr">
         <is>
           <t>Memes dispositions finales que le regime non poste (revision Art. 4.2 ; duree/denonciation 4.1 et 4.3).</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="150" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
+    <row r="11" ht="100.5" customHeight="1">
+      <c r="A11" s="95" t="inlineStr">
         <is>
           <t>Compte Épargne Temps (CET)</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="97" t="n"/>
+      <c r="C11" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="96" t="inlineStr">
         <is>
           <t>19/03/2021</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="97" t="inlineStr">
         <is>
           <t>accord-cet-2021.pdf</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="97" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="97" t="inlineStr">
         <is>
           <t>resume-cet-avenant-2022.md</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="97" t="inlineStr">
         <is>
           <t>Depliant_CET_FO.pdf</t>
         </is>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J11" s="97" t="inlineStr">
         <is>
           <t>PDF de l'accord de base retrouve et integre le 20/10/2026 (David l'a ajoute dans son dossier local). Signatures verifiees visuellement sur le PDF de base (19/03/2021) : ICO (Campone), CGT-FO, CFDT, CFE-CGC ont signe ; Sud Sante-Sociaux (Isabelle Fouillet), partie a l'accord, n'a pas de signature visible sur la page de signature  (même constat pour l'avenant n°1, voir sa ligne). Contenu du .md verifie conforme au PDF signe (preambule, articles 1 a 8, plafonds).</t>
         </is>
       </c>
-      <c r="K11" s="25" t="inlineStr">
+      <c r="K11" s="97" t="inlineStr">
         <is>
           <t>Aucune coquille relevee lors de la relecture.</t>
         </is>
       </c>
-      <c r="L11" s="25" t="inlineStr">
+      <c r="L11" s="97" t="inlineStr">
         <is>
           <t>Bilan quantitatif et qualitatif de l'application de l'accord, presente chaque annee au CSE central (Art. 8.1).</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="150" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
+    <row r="12" ht="100.5" customHeight="1">
+      <c r="A12" s="98" t="n"/>
+      <c r="B12" s="99" t="inlineStr">
         <is>
           <t>Avenant — CET n°1 (31/01/2022)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="C12" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="100" t="inlineStr">
         <is>
           <t>31/01/2022</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="98" t="inlineStr">
         <is>
           <t>Accord CET_Avenant n1_signé.pdf</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="98" t="inlineStr">
         <is>
           <t>manquant (version de travail Word convertie en .md : Accord_CET_Avenant_n_1_vDéfinitive)</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="98" t="inlineStr">
         <is>
           <t>resume-cet-avenant-2022.md</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="98" t="inlineStr">
         <is>
           <t>Depliant_CET_FO.pdf</t>
         </is>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="98" t="inlineStr">
         <is>
           <t>Ligne séparée le 20/10/2026. Annule et remplace l'art. 3.3 (alimentation du CET) de l'accord du 19/03/2021 ; date limite de dépôt des éléments temporels fixée au 15 janvier. Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). Mis à la signature du 31/01 au 11/02/2022. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
-      <c r="K12" s="25" t="inlineStr">
+      <c r="K12" s="98" t="inlineStr">
         <is>
           <t>Art. 'l'artice 3' au lieu de 'l'article 3' (faute de frappe), relevée auparavant sur la ligne de l'accord ATT non cadres : à revérifier sur le texte du PDF.</t>
         </is>
       </c>
-      <c r="L12" s="25" t="inlineStr">
+      <c r="L12" s="98" t="inlineStr">
         <is>
           <t>Durée indéterminée ; entrée en vigueur le lendemain du dépôt (art. 2.1). Pas de suivi propre à l'avenant (le bilan annuel de l'accord de base, art. 8.1, continue de s'appliquer).</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="75" customHeight="1">
-      <c r="A13" s="27" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="95" t="inlineStr">
         <is>
           <t>CDD à objet défini</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="92" t="n"/>
+      <c r="C13" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="96" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="97" t="inlineStr">
         <is>
           <t>Accord CDD à objet défini_Signé.pdf</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="97" t="inlineStr">
         <is>
           <t>Accord CDD à objet défini_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G13" s="97" t="inlineStr">
         <is>
           <t>resume-cdd-objet-defini-2021.md</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H13" s="97" t="inlineStr">
         <is>
           <t>Depliant_CDD_objet_defini_FO.pdf</t>
         </is>
       </c>
-      <c r="I13" s="10" t="n">
+      <c r="I13" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J13" s="8" t="n"/>
-      <c r="K13" s="25" t="inlineStr">
+      <c r="J13" s="97" t="n"/>
+      <c r="K13" s="97" t="inlineStr">
         <is>
           <t>Art. 3 : 'se substitute' au lieu de 'se substitue' (faute). Art. 6.4 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 13/08/2021, DIRECCTE supprimee en avril 2021).</t>
         </is>
       </c>
-      <c r="L13" s="25" t="inlineStr">
+      <c r="L13" s="97" t="inlineStr">
         <is>
           <t>Information du CSE central a chaque conclusion/fin de contrat (Art. 6.1) ; duree indeterminee (6.2) ; revision et denonciation (6.3/6.4).</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="26" t="inlineStr">
+    <row r="14" ht="87" customHeight="1">
+      <c r="A14" s="95" t="inlineStr">
         <is>
           <t>PERCOL (épargne retraite collective)</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="92" t="n"/>
+      <c r="C14" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="96" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="97" t="inlineStr">
         <is>
           <t>Accord PERCOL_Signé.pdf</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="97" t="inlineStr">
         <is>
           <t>Accord PERCOL_vDéfinitive.docx</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="97" t="inlineStr">
         <is>
           <t>resume-percol-2021.md</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="97" t="inlineStr">
         <is>
           <t>Depliant_PERCOL_FO.pdf</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I14" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="25" t="inlineStr">
+      <c r="J14" s="97" t="n"/>
+      <c r="K14" s="97" t="inlineStr">
         <is>
           <t>Orthographe incoherente du nom d'une signataire dans le meme document : 'Genevieve' (preambule) vs 'Genevieve' sans accent (signatures). DIRECCTE correcte pour sa date (19/03/2021, avant le changement d'avril 2021).</t>
         </is>
       </c>
-      <c r="L14" s="25" t="inlineStr">
+      <c r="L14" s="97" t="inlineStr">
         <is>
           <t>Conseils de surveillance des FCPE reunis au moins 1x/an, rapport annuel de gestion (Art. 8) ; information periodique du personnel, communication annuelle de l'epargne (Art. 7) ; revision par avenant (10) ; duree indeterminee et denonciation avec preavis de 3 mois (6) ; procedure de reglement amiable des litiges (11).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="165" customHeight="1">
-      <c r="A15" s="27" t="inlineStr">
+    <row r="15" ht="114" customHeight="1">
+      <c r="A15" s="95" t="inlineStr">
         <is>
           <t>Congé humanitaire</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="92" t="n"/>
+      <c r="C15" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D15" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="97" t="inlineStr">
         <is>
           <t>Accord Congé Humanitaire (2026).pdf</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F15" s="97" t="inlineStr">
         <is>
           <t>Accord sur le congé humanitaire V2.docx</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G15" s="97" t="inlineStr">
         <is>
           <t>resume-conge-humanitaire-2026.md</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="H15" s="97" t="inlineStr">
         <is>
           <t>Depliant_conge_humanitaire_FO.pdf</t>
         </is>
       </c>
-      <c r="I15" s="10" t="n">
+      <c r="I15" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="8" t="n"/>
-      <c r="K15" s="25" t="inlineStr">
+      <c r="J15" s="97" t="n"/>
+      <c r="K15" s="97" t="inlineStr">
         <is>
           <t>Numerotation incoherente des dispositions finales : l'Art. 7.3 'Formalites de depot et publicite' traite en realite de la denonciation ; l'Art. 7.4 porte le meme intitule mais traite, lui, du vrai depot -- il manque un intitule '7.3 Denonciation'. Art. 1 : 'LeS beneficiaires' (casse) et 'beneficie d'un conge' au lieu de 'benefice' (faute). Art. 7.3 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 31/03/2026).</t>
         </is>
       </c>
-      <c r="L15" s="25" t="inlineStr">
+      <c r="L15" s="97" t="inlineStr">
         <is>
           <t>Consultation du CSE de rattachement en cas de refus d'une demande 'ordinaire' (Art. 3.1, non requise pour l'urgence humanitaire 3.2) ; revision (7.2) ; duree indeterminee et denonciation (7.1 et 7.3, referencee par son numero reel malgre l'intitule errone).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="210" customHeight="1">
-      <c r="A16" s="26" t="inlineStr">
+    <row r="16" ht="141" customHeight="1">
+      <c r="A16" s="95" t="inlineStr">
         <is>
           <t>Égalité femmes-hommes</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="92" t="n"/>
+      <c r="C16" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="96" t="inlineStr">
         <is>
           <t>2026 (version en vigueur)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="97" t="inlineStr">
         <is>
           <t>Accord égalité FH 2026.pdf</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="97" t="inlineStr">
         <is>
           <t>Accord Egalité F H_V2026 05 20.docx</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="97" t="inlineStr">
         <is>
           <t>resume-egalite-fh-2026.md</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="97" t="inlineStr">
         <is>
           <t>Depliant_egalite_femmes_hommes_FO.pdf</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I16" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="25" t="inlineStr">
+      <c r="J16" s="97" t="n"/>
+      <c r="K16" s="97" t="inlineStr">
         <is>
           <t>Numerotation d'article dupliquee : deux 'Article 8' distincts (violences domestiques, puis dispositions finales) avec un sous-numero '8.1' utilise deux fois pour des sujets differents. CONFIRME COQUILLE PAR DAVID DI PERI LE 20/10/2026 : contradiction Art. 7.4 entre le corps de l'article (conge de parentalite homoparental accorde a un seul des deux membres du couple si les 2 sont salaries de l'ICO) et le tableau juste en dessous (qui semble l'attribuer aux deux dans la 1ere situation) -- erreur de redaction, le corps de l'article fait foi.</t>
         </is>
       </c>
-      <c r="L16" s="25" t="inlineStr">
+      <c r="L16" s="97" t="inlineStr">
         <is>
           <t>Bilan annuel quantitatif/qualitatif au CSE central, clause de revoyure apres la 1ere annee (Art. 8 Dispositions finales) ; suivi specifique des violences domestiques -- etat statistique annuel en commission Formation Egalite FH (8.2.4).</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="90" customHeight="1">
-      <c r="A17" s="27" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="95" t="inlineStr">
         <is>
           <t>Travail de nuit</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="92" t="n"/>
+      <c r="C17" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D17" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E17" s="97" t="inlineStr">
         <is>
           <t>Accord travail de nuit - 2026.pdf</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="97" t="inlineStr">
         <is>
           <t>Accord  nuit V 2026 05 04.docx</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G17" s="97" t="inlineStr">
         <is>
           <t>resume-travail-nuit-2026.md</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" s="97" t="inlineStr">
         <is>
           <t>Depliant_stages_de_jour_personnel_nuit_FO.pdf</t>
         </is>
       </c>
-      <c r="I17" s="10" t="n">
+      <c r="I17" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J17" s="8" t="n"/>
-      <c r="K17" s="25" t="inlineStr">
+      <c r="J17" s="97" t="n"/>
+      <c r="K17" s="97" t="inlineStr">
         <is>
           <t>'certains activites' au lieu de 'certaines activites' (accord grammatical fautif, faute mineure).</t>
         </is>
       </c>
-      <c r="L17" s="25" t="inlineStr">
+      <c r="L17" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, entree en vigueur 01/08/2026 (Art. 3.1) ; revision (3.2) ; denonciation avec preavis de 3 mois, effets sur 1 an (3.3). Aucun mecanisme de suivi/commission/bilan prevu par cet accord.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="255" customHeight="1">
-      <c r="A18" s="26" t="inlineStr">
+    <row r="18" ht="168" customHeight="1">
+      <c r="A18" s="95" t="inlineStr">
         <is>
           <t>Validation des Acquis Professionnels (VAP)</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="97" t="n"/>
+      <c r="C18" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="96" t="inlineStr">
         <is>
           <t>22/03/2024</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="97" t="inlineStr">
         <is>
           <t>Accord sur la validation des acquis professionnels _Version signée.pdf</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="97" t="inlineStr">
         <is>
           <t>Accord sur la validation des acquis professionnels V2025-2.docx</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="97" t="inlineStr">
         <is>
           <t>resume-vap-2025.md</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="97" t="inlineStr">
         <is>
           <t>Depliant_VAP_FO.pdf</t>
         </is>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I18" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J18" s="97" t="inlineStr">
         <is>
           <t>Avenant du 04/02/2025 désormais sur sa propre ligne (voir 'Avenant — VAP'). PDF signe (22/03/2024, 'Accord VAP - V2') verifie visuellement page par page le 20/10/2026 : signe ICO (Pr Campone, DG), CGT-FO (David Di Peri), CFE-CGC (Maxime Bremaud). AUCUNE signature ni paraphe de Sud Sante-Sociaux (Julien Rosan) sur les 5 pages -- ce syndicat n'a pas signe l'accord de base.</t>
         </is>
       </c>
-      <c r="K18" s="25" t="inlineStr">
+      <c r="K18" s="97" t="inlineStr">
         <is>
           <t>Acronyme errone 'DDRETS' (Art. 3.3, Denonciation) -- n'existe pas (DREETS regionale ou DDETS departementale), present a l'identique dans le brouillon .md et dans le PDF reellement signe de l'avenant. A RECLASSER : le fichier .md stocke a cote de ce PDF sous le nom 'Accord sur la validation des acquis professionnels _Version signee.md' contient en realite le texte de l'AVENANT 2025 (V2025-2), pas celui de l'accord de base 22/03/2024. Aucune conversion Markdown du vrai accord de base (PDF 'Version signee', 22/03/2024) n'existe a ce jour -- a produire separement. Decision de David 20/10/2026 : ne retenir que le PDF signe comme reference, pas le brouillon Word.</t>
         </is>
       </c>
-      <c r="L18" s="25" t="inlineStr">
+      <c r="L18" s="97" t="inlineStr">
         <is>
           <t>Aucun mecanisme de suivi identifie (ni commission, ni bilan, ni indicateur) -- seules duree, revision, denonciation, depot sont prevues.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="225" customHeight="1">
-      <c r="A19" s="27" t="inlineStr">
+    <row r="19" ht="141" customHeight="1">
+      <c r="A19" s="98" t="n"/>
+      <c r="B19" s="99" t="inlineStr">
         <is>
           <t>Avenant — VAP (04/02/2025)</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="C19" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="100" t="inlineStr">
         <is>
           <t>04/02/2025</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E19" s="98" t="inlineStr">
         <is>
           <t>Avenant à l'accord d'entreprise relatif à la Validation des Acquis Professionnels _04.02.2025_0.pdf</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="98" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="G19" s="98" t="inlineStr">
         <is>
           <t>resume-vap-2025.md</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="98" t="inlineStr">
         <is>
           <t>Depliant_VAP_FO.pdf</t>
         </is>
       </c>
-      <c r="I19" s="10" t="n">
+      <c r="I19" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="J19" s="98" t="inlineStr">
         <is>
           <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Confirmé : porte l'étiquette V2025-2, cohérente avec le Word conservé. PDF signe (04/02/2025, 'Avenant accord VAP V2025-2') verifie visuellement page par page le 20/10/2026 : signe CFE-CGC (Maxime Bremaud), CGT-FO par delegation (Mme Le Guillou 'P/ D. Di Peri'), Sud Sante-Sociaux (Julien Rosan). AUCUNE signature ni paraphe de l'ICO/Direction Generale (Pr Campone) sur les 4 pages, alors que son nom figure dans l'en-tete des signataires -- a clarifier avec la Direction.</t>
         </is>
       </c>
-      <c r="K19" s="25" t="inlineStr">
+      <c r="K19" s="98" t="inlineStr">
         <is>
           <t>CLASSEMENT DOCUMENTAIRE ERRONE (confirme) : le fichier utilise comme 'accord de base' VAP est en realite le brouillon de cet avenant, avec des dates incoherentes avec le PDF reellement signe (brouillon : 'Fait le 25/02/2025' ; PDF signe : 'Fait le 4 fevrier 2025'). Decision de David 20/10/2026 : ne retenir que le PDF signe comme reference -- resume corrige en consequence le 20/10/2026 (date et signatures reprises du PDF uniquement). Meme coquille 'DDRETS' (au lieu de DREETS/DDETS) reproduite dans le brouillon et dans le PDF signe (Art. 3.3, Denonciation).</t>
         </is>
       </c>
-      <c r="L19" s="25" t="inlineStr">
+      <c r="L19" s="98" t="inlineStr">
         <is>
           <t>Aucun mecanisme de suivi identifie.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="90" customHeight="1">
-      <c r="A20" s="26" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="95" t="inlineStr">
         <is>
           <t>Répartition de la BIC</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="92" t="n"/>
+      <c r="C20" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="96" t="inlineStr">
         <is>
           <t>2025 (V2025-2)</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" s="97" t="inlineStr">
         <is>
           <t>Accord relatif à la répartition de la BIC_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="97" t="inlineStr">
         <is>
           <t>Accord sur la répartition de la BIC V2025-2.docx</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="97" t="inlineStr">
         <is>
           <t>resume-bic-2025.md</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="97" t="inlineStr">
         <is>
           <t>Depliant_BIC_FO.pdf</t>
         </is>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I20" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="25" t="inlineStr">
+      <c r="J20" s="97" t="n"/>
+      <c r="K20" s="97" t="inlineStr">
         <is>
           <t>Art. 1 : 'valorisaiton' au lieu de 'valorisation' (faute). Art. 3.3 : 'DDRETS d'Angers' -- sigle inexistant (devrait etre DREETS).</t>
         </is>
       </c>
-      <c r="L20" s="25" t="inlineStr">
+      <c r="L20" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, entree en vigueur le 1er jour du mois suivant le depot (Art. 3.1) ; revision sous 2 mois (3.2) ; denonciation par LRAR (3.3). Aucune commission de suivi, bilan ou indicateur specifique prevu.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="285" customHeight="1">
-      <c r="A21" s="27" t="inlineStr">
+    <row r="21" ht="195" customHeight="1">
+      <c r="A21" s="95" t="inlineStr">
         <is>
           <t>Intéressement</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="92" t="n"/>
+      <c r="C21" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="96" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E21" s="97" t="inlineStr">
         <is>
           <t>Accord d'entreprise relatif à l'intéressement (2026).pdf</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F21" s="97" t="inlineStr">
         <is>
           <t>Accord  intéressement 2026 _ Version 4 (22.05.2026).docx</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G21" s="97" t="inlineStr">
         <is>
           <t>resume-interessement-2026.md</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H21" s="97" t="inlineStr">
         <is>
           <t>Depliant_interessement_FO.pdf</t>
         </is>
       </c>
-      <c r="I21" s="10" t="n">
+      <c r="I21" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="25" t="inlineStr">
+      <c r="J21" s="97" t="n"/>
+      <c r="K21" s="97" t="inlineStr">
         <is>
           <t>Titre Art. 4 : 'INTESSEMENT' (faute dans le titre). Art. 4 annonce 'quatre indicateurs' mais seuls trois sont definis et utilises dans la formule finale I = SG+AV+CAF. Art. 4.1 (bareme E-Satis, classe B, x2) : '75 0000 EUR' au lieu de 75 000 EUR. Art. 8.1 : 'Comite Sociale et Economique' (faute d'accord). CONFIRME COQUILLE PAR DAVID DI PERI LE 20/10/2026 : le Preambule annonce le dispositif pour 2026-2027-2028, mais l'Art. 9.1 (texte normatif) fixe une duree limitee a l'exercice 2026 seul -- erreur de redaction au preambule ; a defaut d'avenant, 2027 et 2028 devront faire l'objet d'un nouvel accord. Signale dans le resume. Art. 7.1 : ambiguite entre 'dernier jour du mois suivant la cloture de l'exercice' et la date donnee '31 mai N+1'.</t>
         </is>
       </c>
-      <c r="L21" s="25" t="inlineStr">
+      <c r="L21" s="97" t="inlineStr">
         <is>
           <t>Suivi par le CSE central a chaque calcul/repartition (Art. 8.1) ; bilan annuel presente en CSE central (8.1) ; fiche individuelle pour chaque salarie (8.2) ; clause de revoyure si la HAS modifie un indicateur (4.1) ; negociation obligatoire avant tout supplement d'interessement (4.3) ; procedure de reglement des differends + bilan annuel des litiges en NAO (9.2) ; revision (9.3) ; denonciation (9.4).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="105" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
+    <row r="22" ht="73.5" customHeight="1">
+      <c r="A22" s="95" t="inlineStr">
         <is>
           <t>Forfait Mobilité Durable</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="92" t="n"/>
+      <c r="C22" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="96" t="inlineStr">
         <is>
           <t>24/10/2025</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" s="97" t="inlineStr">
         <is>
           <t>Accord Forfait Mobilite Durable 2025 signe.pdf</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="97" t="inlineStr">
         <is>
           <t>Accord Forfait Mobilité Durable Vfinale.docx</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G22" s="97" t="inlineStr">
         <is>
           <t>resume-forfait-mobilite-durable-2025.md</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H22" s="97" t="inlineStr">
         <is>
           <t>Depliant_forfait_mobilite_durable_FO.pdf</t>
         </is>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I22" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J22" s="97" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant) : daté du 24/10/2025, signé DG/CGT-FO/CFE-CGC. ⚠️ Sud Santé-Sociaux n'a pas signé (ligne vide). 20/10/2026 : doublon du PDF non signé supprimé, le lien du résumé pointe vers « signe.pdf ». Signataires du dépliant : DG, CGT-FO et CFE-CGC.</t>
         </is>
       </c>
-      <c r="K22" s="25" t="inlineStr">
+      <c r="K22" s="97" t="inlineStr">
         <is>
           <t>Art. 6.3 (Denonciation) : 'DIRECCTE d'Angers' -- anachronisme (accord signe 24/10/2025).</t>
         </is>
       </c>
-      <c r="L22" s="25" t="inlineStr">
+      <c r="L22" s="97" t="inlineStr">
         <is>
           <t>Revision (Art. 6.2) ; duree indeterminee et denonciation liee aux mandats CSE (6.1 et 6.3). Pas de commission de suivi/bilan prevu par l'accord lui-meme ; le dispositif a toutefois deja ete revu deux fois par la voie des NAO (2024 puis 2025).</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
+    <row r="23" ht="46.5" customHeight="1">
+      <c r="A23" s="95" t="inlineStr">
         <is>
           <t>Prime chaussures</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="92" t="n"/>
+      <c r="C23" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="96" t="inlineStr">
         <is>
           <t>21/06/2023</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="97" t="inlineStr">
         <is>
           <t>Accord prime chaussure version signée.pdf</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="97" t="inlineStr">
         <is>
           <t>Accord Prime Chaussures V finale.docx</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G23" s="97" t="inlineStr">
         <is>
           <t>resume-prime-chaussures-2023.md</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H23" s="97" t="inlineStr">
         <is>
           <t>Depliant_prime_chaussures_FO.pdf</t>
         </is>
       </c>
-      <c r="I23" s="10" t="n">
+      <c r="I23" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J23" s="8" t="n"/>
-      <c r="K23" s="25" t="inlineStr">
+      <c r="J23" s="97" t="n"/>
+      <c r="K23" s="97" t="inlineStr">
         <is>
           <t>Art. 4.3 : 'DREET d'Angers' -- lettre 'S' manquante (devrait etre DREETS).</t>
         </is>
       </c>
-      <c r="L23" s="25" t="inlineStr">
+      <c r="L23" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee depuis le 01/07/2023 (Art. 4.1) ; revision sous 2 mois (4.2) ; denonciation par LRAR (4.3). Aucune commission de suivi ni bilan specifique.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="255" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
+    <row r="24" ht="168" customHeight="1">
+      <c r="A24" s="95" t="inlineStr">
         <is>
           <t>Prime USC</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="97" t="n"/>
+      <c r="C24" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="96" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" s="97" t="inlineStr">
         <is>
           <t>Accord prime USC signé.pdf</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="97" t="inlineStr">
         <is>
           <t>Accord prime USC V finale.docx</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="97" t="inlineStr">
         <is>
           <t>resume-prime-usc-2023.md</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H24" s="97" t="inlineStr">
         <is>
           <t>Depliant_prime_USC_FO.pdf</t>
         </is>
       </c>
-      <c r="I24" s="6" t="n">
+      <c r="I24" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J24" s="97" t="inlineStr">
         <is>
           <t>Avenant du 26/04/2024 désormais sur sa propre ligne (voir 'Avenant — Prime USC'). 20/10/2026 : résumé et dépliant mis à jour (avenant du 26/04/2024 intégré, contexte retiré).</t>
         </is>
       </c>
-      <c r="K24" s="25" t="inlineStr">
+      <c r="K24" s="97" t="inlineStr">
         <is>
           <t>Preambule : incoherence temporelle ('deploye sur l'annee 2022' vs effet 'a compter du 1er janvier 2023'). Art. 2 : 'soins continue' et 'est arretee' -- fautes d'accord (devrait etre 'soins continu', 'est arrete'). Art. 3.2 (x2) : 'bruits' au lieu de 'bruts'. A CORRIGER DANS LE RESUME : Art. 3.3 -- erreur de notation mathematique, le texte ecrit '(130/80%=104)' (symbole division) alors que l'operation reelle est une multiplication (130x80%=104) ; le resultat chiffre est juste mais le symbole est faux, et cette formule erronee est reprise telle quelle dans le resume actuel. Art. 4.3 : 'DIRECCTE d'Angers' -- anachronisme (accord signe decembre 2023).</t>
         </is>
       </c>
-      <c r="L24" s="25" t="inlineStr">
+      <c r="L24" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, effet retroactif au 01/01/2023 (Art. 4.1) ; revision sous 2 mois (4.2) ; denonciation par LRAR (4.3). Aucune commission de suivi ni bilan specifique.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="165" customHeight="1">
-      <c r="A25" s="27" t="inlineStr">
+    <row r="25" ht="114" customHeight="1">
+      <c r="A25" s="98" t="n"/>
+      <c r="B25" s="99" t="inlineStr">
         <is>
           <t>Avenant — Prime USC (26/04/2024)</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="C25" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="100" t="inlineStr">
         <is>
           <t>26/04/2024</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="98" t="inlineStr">
         <is>
           <t>AVENANT ACCORD PRIME USC_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F25" s="98" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="G25" s="98" t="inlineStr">
         <is>
           <t>resume-prime-usc-2023.md</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="H25" s="98" t="inlineStr">
         <is>
           <t>Depliant_prime_USC_FO.pdf</t>
         </is>
       </c>
-      <c r="I25" s="10" t="n">
+      <c r="I25" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="J25" s="8" t="inlineStr">
+      <c r="J25" s="98" t="inlineStr">
         <is>
           <t>Ligne créée le 19/10/2026. Aucun Word reçu. Transcription Markdown ajoutée le 20/10/2026 (« AVENANT ACCORD PRIME USC_Version signee.md », relue visuellement contre le PDF). Contenu intégré au résumé et au dépliant : art. 1 (règle d'au moins 50 % de nuits pour les IDE et AS de nuit de Saint-Herblain), art. 2 (règle future après ouverture d'Ambicion / USIP). ⚠️ Point à trancher par David : lecture de la formule applicable après l'ouverture d'Ambicion / USIP (le texte renvoie aux collègues de jour ou d'Angers).</t>
         </is>
       </c>
-      <c r="K25" s="25" t="inlineStr">
+      <c r="K25" s="98" t="inlineStr">
         <is>
           <t>Voir ligne Prime USC (coquille « 130/80 % = 104 » à l'art. 3.3 de l'accord de base).</t>
         </is>
       </c>
-      <c r="L25" s="25" t="n"/>
-    </row>
-    <row r="26" ht="75" customHeight="1">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="L25" s="98" t="n"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="95" t="inlineStr">
         <is>
           <t>PVA</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="92" t="n"/>
+      <c r="C26" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="96" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="97" t="inlineStr">
         <is>
           <t>Accord PVA_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="97" t="inlineStr">
         <is>
           <t>Accord PVA_vFinale.docx</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="97" t="inlineStr">
         <is>
           <t>resume-pva-2022.md</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H26" s="97" t="inlineStr">
         <is>
           <t>Depliant_PVA_FO.pdf</t>
         </is>
       </c>
-      <c r="I26" s="6" t="n">
+      <c r="I26" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="25" t="inlineStr">
+      <c r="J26" s="97" t="n"/>
+      <c r="K26" s="97" t="inlineStr">
         <is>
           <t>Art. 8.4 (Denonciation) : 'DIRECCTE d'Angers' -- anachronisme (accord signe mai 2022). Aucune autre coquille relevee (numerotation 1 a 8 coherente).</t>
         </is>
       </c>
-      <c r="L26" s="25" t="inlineStr">
+      <c r="L26" s="97" t="inlineStr">
         <is>
           <t>Indicateurs de suivi par service communiques chaque annee au CSE central (Art. 7) ; bilan annuel qualitatif/quantitatif au CSE central (8.1) ; clause de revoyure apres la 1ere annee (8.1).</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="120" customHeight="1">
-      <c r="A27" s="27" t="inlineStr">
+    <row r="27" ht="87" customHeight="1">
+      <c r="A27" s="101" t="inlineStr">
         <is>
           <t>Prime de retour inopiné (DUE, non négociée)</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="92" t="n"/>
+      <c r="C27" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="D27" s="102" t="inlineStr">
         <is>
           <t>01/05/2024 (DUE, non négociée)</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E27" s="103" t="inlineStr">
         <is>
           <t>DUE_Prime de retour inopiné.pdf</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="103" t="inlineStr">
         <is>
           <t>DUE_Prime de retour inopiné 01.05.2024 _ MER IDE AS.docx</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="G27" s="103" t="inlineStr">
         <is>
           <t>resume-prime-retour-inopine.md</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="H27" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_retour_inopine_FO.pdf</t>
         </is>
       </c>
-      <c r="I27" s="10" t="n">
+      <c r="I27" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="8" t="n"/>
-      <c r="K27" s="25" t="inlineStr">
+      <c r="J27" s="103" t="n"/>
+      <c r="K27" s="103" t="inlineStr">
         <is>
           <t>Point 3 : 'Des lors que' -- accent manquant sur 'Des' (orthographe). Ambiguite entre le point 4 (prime applicable aux AS/IDE 'depuis la premiere DUE de fevrier 2023') et le point 6 ('prise a effet du 1er mai 2024') -- pas de distinction claire de la date d'effet selon les categories de personnel.</t>
         </is>
       </c>
-      <c r="L27" s="25" t="inlineStr">
+      <c r="L27" s="103" t="inlineStr">
         <is>
           <t>Aucune clause de revision/bilan/commission ; seul un outil de tracabilite administrative (Chronos) est mentionne pour le decompte du temps, pas un controle de l'application de la DUE elle-meme.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="75" customHeight="1">
-      <c r="A28" s="26" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="95" t="inlineStr">
         <is>
           <t>Parcours professionnel — Assistants Médicaux</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="92" t="n"/>
+      <c r="C28" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" s="96" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="97" t="inlineStr">
         <is>
           <t>Accord relatif au parcours des assistantes médicales_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="97" t="inlineStr">
         <is>
           <t>Accord parcours AM Version finale.docx</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G28" s="97" t="inlineStr">
         <is>
           <t>resume-parcours-am-2025.md</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H28" s="97" t="inlineStr">
         <is>
           <t>Depliant_parcours_assistant_medical_FO.pdf</t>
         </is>
       </c>
-      <c r="I28" s="6" t="n">
+      <c r="I28" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="4" t="n"/>
-      <c r="K28" s="25" t="inlineStr">
+      <c r="J28" s="97" t="n"/>
+      <c r="K28" s="97" t="inlineStr">
         <is>
           <t>Art. 4.3 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 11/03/2025).</t>
         </is>
       </c>
-      <c r="L28" s="25" t="inlineStr">
+      <c r="L28" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, entree en vigueur 01/04/2025 (Art. 4.1) ; revision et denonciation (4.2/4.3). Aucun mecanisme specifique (pas de commission de suivi ni bilan annuel).</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="27" t="inlineStr">
+    <row r="29" ht="46.5" customHeight="1">
+      <c r="A29" s="95" t="inlineStr">
         <is>
           <t>Parcours professionnel — IDE / MER</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="92" t="n"/>
+      <c r="C29" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
+      <c r="D29" s="96" t="inlineStr">
         <is>
           <t>13/03/2025</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E29" s="97" t="inlineStr">
         <is>
           <t>Accord parcours IDE et MER_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F29" s="97" t="inlineStr">
         <is>
           <t>Accord parcours IDE et MER V 2025 03 13 - VF.docx</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="G29" s="97" t="inlineStr">
         <is>
           <t>resume-parcours-ide-mer-2025.md</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr">
+      <c r="H29" s="97" t="inlineStr">
         <is>
           <t>Depliant_parcours_IDE_MER_FO.pdf</t>
         </is>
       </c>
-      <c r="I29" s="10" t="n">
+      <c r="I29" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J29" s="8" t="n"/>
-      <c r="K29" s="25" t="inlineStr">
+      <c r="J29" s="97" t="n"/>
+      <c r="K29" s="97" t="inlineStr">
         <is>
           <t>Art. 2-1 : 'ne beneface pas' au lieu de 'ne beneficie pas' (faute). Art. 4.3 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 28/03/2025).</t>
         </is>
       </c>
-      <c r="L29" s="25" t="inlineStr">
+      <c r="L29" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, entree en vigueur 01/05/2025 (Art. 4.1) ; revision et denonciation (4.2/4.3). Aucun mecanisme specifique.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="105" customHeight="1">
-      <c r="A30" s="26" t="inlineStr">
+    <row r="30" ht="73.5" customHeight="1">
+      <c r="A30" s="95" t="inlineStr">
         <is>
           <t>Parcours professionnel — Physiciens médicaux</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="92" t="n"/>
+      <c r="C30" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="96" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="97" t="inlineStr">
         <is>
           <t>Accord Parcours Phycisiens_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="97" t="inlineStr">
         <is>
           <t>Accord Physiciens médicaux 2022_vFinale.docx</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="97" t="inlineStr">
         <is>
           <t>resume-parcours-physiciens-2022.md</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H30" s="97" t="inlineStr">
         <is>
           <t>Depliant_parcours_physiciens_medicaux_FO.pdf</t>
         </is>
       </c>
-      <c r="I30" s="6" t="n">
+      <c r="I30" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J30" s="4" t="n"/>
-      <c r="K30" s="25" t="inlineStr">
+      <c r="J30" s="97" t="n"/>
+      <c r="K30" s="97" t="inlineStr">
         <is>
           <t>CONFIRME : Art. 2, les deux exemples chiffres indiquent qu'un CS2 'sera rattache au groupe L', alors que l'Art. 1 situe explicitement CS2 au Groupe M (Groupe L = CS1) -- incoherence interne a faire remonter a la Direction. Art. 4.3 : 'DREET d'Angers' -- lettre 'S' manquante.</t>
         </is>
       </c>
-      <c r="L30" s="25" t="inlineStr">
+      <c r="L30" s="97" t="inlineStr">
         <is>
           <t>Duree indeterminee, entree en vigueur 01/07/2022 (Art. 4.1) ; revision et denonciation (4.2/4.3). Aucun mecanisme specifique (l'Art. 3 ne fixe qu'une date de bascule DUE-&gt;accord, pas un dispositif de suivi).</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="75" customHeight="1">
-      <c r="A31" s="27" t="inlineStr">
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="95" t="inlineStr">
         <is>
           <t>Reprise d'ancienneté — MER / AS / IDE</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="92" t="n"/>
+      <c r="C31" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D31" s="10" t="inlineStr">
+      <c r="D31" s="96" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E31" s="97" t="inlineStr">
         <is>
           <t>Accord Reprise Expérience professionnelle MER-AS-IDE_2022_Signé.pdf</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
+      <c r="F31" s="97" t="inlineStr">
         <is>
           <t>Accord reprise ancienneté MER IDE AS_vFinale.docx</t>
         </is>
       </c>
-      <c r="G31" s="8" t="inlineStr">
+      <c r="G31" s="97" t="inlineStr">
         <is>
           <t>resume-reprise-anciennete-mer-as-ide-2022.md</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr">
+      <c r="H31" s="97" t="inlineStr">
         <is>
           <t>Depliant_reprise_anciennete_MER_IDE_AS_FO.pdf</t>
         </is>
       </c>
-      <c r="I31" s="10" t="n">
+      <c r="I31" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J31" s="8" t="n"/>
-      <c r="K31" s="25" t="inlineStr">
+      <c r="J31" s="97" t="n"/>
+      <c r="K31" s="97" t="inlineStr">
         <is>
           <t>Saut de numerotation : le document passe de l'Article 4 (4-1, 4-2) a l'Article 6 -- il n'existe pas d'Article 5. Art. 6.4 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 19/05/2022).</t>
         </is>
       </c>
-      <c r="L31" s="25" t="inlineStr">
+      <c r="L31" s="97" t="inlineStr">
         <is>
           <t>Suivi organise dans le cadre du CSE central avant fin 2022, communication du nombre de salaries ayant demande la reprise a 100% (Art. 6.1).</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="330" customHeight="1">
-      <c r="A32" s="26" t="inlineStr">
+    <row r="32" ht="222" customHeight="1">
+      <c r="A32" s="104" t="inlineStr">
         <is>
           <t>Dialogue social</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="92" t="n"/>
+      <c r="C32" s="105" t="inlineStr">
         <is>
           <t>Élections</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="105" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" s="106" t="inlineStr">
         <is>
           <t>Accord dialogue social 2026.pdf</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="106" t="inlineStr">
         <is>
           <t>Accord sur le dialogue social 2026_Version 03.docx</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="106" t="inlineStr">
         <is>
           <t>resume-dialogue-social-2026.md</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H32" s="106" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="I32" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J32" s="106" t="inlineStr">
         <is>
           <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
-      <c r="K32" s="25" t="inlineStr">
+      <c r="K32" s="106" t="inlineStr">
         <is>
           <t>Audit repris le 20/10/2026 (David confirme n'avoir jamais demande l'arret de la verification). Coquilles relevees : (1) Art. 1.1 - le premier sous-point 'La fixation de l'ordre du jour' n'est pas numerote 1.1.1 (numerotation commence directement a 1.1.2 'Le lieu de reunion') ; (2) Art. 4.3 renvoie a tort a 'l'article 1.1.9.1' pour le budget de fonctionnement des CSE locaux -- la section reelle est 1.1.8.1 ; (3) Art. 5.3 et Art. 5.4 portent le MEME titre 'Formalites de depot et publicite' alors que le 5.3 traite en realite de la denonciation (pas des formalites de depot) ; (4) Art. 1.2.1, derniere phrase : 'CCSCT' au lieu de 'CSSCT' (faute de frappe) ; (5) Art. 5.3 utilise le terme obsolete 'DIRECCTE d'Angers' (renommee DREETS/DDETS depuis avril 2021 -- meme anomalie deja relevee dans au moins 8 autres accords ICO posterieurs a cette date).</t>
         </is>
       </c>
-      <c r="L32" s="25" t="inlineStr">
+      <c r="L32" s="106" t="inlineStr">
         <is>
           <t>Revision (Art. 5.2, procedure legale L.2261-7-1) ; denonciation (Art. 5.3, LRAR, effets jusqu'au dernier jour des mandats CSE, accord indivisible) ; publicite (Art. 5.4, TeleAccords + greffe CPH Angers + intranet). Aucune commission de suivi, bilan annuel ni indicateur specifique prevu par cet accord.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="135" customHeight="1">
-      <c r="A33" s="27" t="inlineStr">
+    <row r="33" ht="87" customHeight="1">
+      <c r="A33" s="104" t="inlineStr">
         <is>
           <t>Vote électronique</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="92" t="n"/>
+      <c r="C33" s="105" t="inlineStr">
         <is>
           <t>Élections</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
+      <c r="D33" s="105" t="inlineStr">
         <is>
           <t>09/04/2026</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E33" s="106" t="inlineStr">
         <is>
           <t>ACCORD VOTE ELECTRONIQUE _ Elections professionnelles 2026.pdf</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F33" s="106" t="inlineStr">
         <is>
           <t>Accord Vote électronique_v2026 04 09.docx</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
+      <c r="G33" s="106" t="inlineStr">
         <is>
           <t>resume-vote-electronique-2026.md</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr">
+      <c r="H33" s="106" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I33" s="10" t="n">
+      <c r="I33" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="8" t="inlineStr">
+      <c r="J33" s="106" t="inlineStr">
         <is>
           <t>⚠️ Retiré du catalogue/site le 19/10/2026 (toutes pages) sur demande — document source conservé dans docs/elections/, non supprimé. PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
-      <c r="K33" s="25" t="inlineStr">
+      <c r="K33" s="106" t="inlineStr">
         <is>
           <t>Audit repris le 20/10/2026 (David confirme n'avoir jamais demande l'arret de la verification). Aucune coquille relevee dans le corps de l'accord (numerotation 1-6 coherente, pas d'incoherence de fond identifiee). Date de signature deja confirmee sur PDF (29/05/2026) -- le Word source laissait la date en blanc, deja signale.</t>
         </is>
       </c>
-      <c r="L33" s="25" t="inlineStr">
+      <c r="L33" s="106" t="inlineStr">
         <is>
           <t>Revision (Art. 4, modalites du code du travail) ; duree determinee liee aux elections 2026, l'accord cesse de produire effet des l'election definitive des representants (Art. 5) ; publicite (Art. 6, TeleAccords + greffe CPH Angers). Aucune commission de suivi, bilan ou indicateur specifique prevu.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="26" t="inlineStr">
+    <row r="34" ht="46.5" customHeight="1">
+      <c r="A34" s="101" t="inlineStr">
         <is>
           <t>DUE : parcours techniciens de laboratoire / macroscopie</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="92" t="n"/>
+      <c r="C34" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="102" t="inlineStr">
         <is>
           <t>DUE, non datée précisément</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" s="103" t="inlineStr">
         <is>
           <t>DUE Parcours techs de laboratoire-macroscopie_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="103" t="inlineStr">
         <is>
           <t>DUE Tech de labo d'anapath.docx</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="103" t="inlineStr">
         <is>
           <t>resume-due-parcours-macroscopie.md</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H34" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_parcours_macroscopie_FO.pdf</t>
         </is>
       </c>
-      <c r="I34" s="6" t="n">
+      <c r="I34" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J34" s="4" t="n"/>
-      <c r="K34" s="25" t="inlineStr">
+      <c r="J34" s="103" t="n"/>
+      <c r="K34" s="103" t="inlineStr">
         <is>
           <t>Point 1 : 'cycle de de formation' -- mot repete par erreur. Redondance non bloquante (duree du cycle enoncee deux fois).</t>
         </is>
       </c>
-      <c r="L34" s="25" t="inlineStr">
+      <c r="L34" s="103" t="inlineStr">
         <is>
           <t>Aucun mecanisme identifie (ni commission, ni bilan, ni indicateur, ni clause de revision/duree limitee) -- DUE non negociee.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="225" customHeight="1">
-      <c r="A35" s="27" t="inlineStr">
+    <row r="35" ht="141" customHeight="1">
+      <c r="A35" s="101" t="inlineStr">
         <is>
           <t>DUE : complémentaire frais de santé</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B35" s="92" t="n"/>
+      <c r="C35" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D35" s="102" t="inlineStr">
         <is>
           <t>19/06/2024 (DUE)</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="103" t="inlineStr">
         <is>
           <t>DUE regime frais de sante 2024.pdf</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F35" s="103" t="inlineStr">
         <is>
           <t>DUE CFS_v2024 05 27.docx</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
+      <c r="G35" s="103" t="inlineStr">
         <is>
           <t>resume-due-complementaire-frais-sante.md</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
+      <c r="H35" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_complementaire_frais_sante_FO.pdf</t>
         </is>
       </c>
-      <c r="I35" s="10" t="n">
+      <c r="I35" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="8" t="inlineStr">
+      <c r="J35" s="103" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : PDF signé retrouvé le 19/10/2026 (était manquant) — date réelle de signature 19/06/2024, PAS 27/05/2024 comme précédemment indiqué (27/05 était la date du Word, pas de la signature).</t>
         </is>
       </c>
-      <c r="K35" s="25" t="inlineStr">
+      <c r="K35" s="103" t="inlineStr">
         <is>
           <t>Incoherence de date entre le corps (signee 'le 19 juin 2024') et le coupon-reponse (mentionne une decision 'datee du 1er juin 2024') -- confusion entre date de signature et date d'effet du regime. Art. 3 : les dispenses n5/6 (art. R.242-1-6) reprennent presque mot pour mot les dispenses n1/2 (L.911-7 III/D.911-2) sans que la difference pratique soit clairement expliquee. | Un regime anterieur (2022, scinde cadre/non cadre) portait par erreur le titre 'Prevoyance' alors qu'il s'agit du meme regime frais de sante -- voir dossier prevoyance-mutuelle-retraite.</t>
         </is>
       </c>
-      <c r="L35" s="25" t="inlineStr">
+      <c r="L35" s="103" t="inlineStr">
         <is>
           <t>Notice d'information remise a chaque salarie, modifications communiquees de meme (Art. 9) ; information-consultation du CSE avant toute mise en place ou modification du regime (10) ; duree indeterminee, modification/denonciation possible par l'employeur selon la procedure des engagements unilateraux -- pas de revision negociee, DUE (11).</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="120" customHeight="1">
-      <c r="A36" s="26" t="inlineStr">
+    <row r="36" ht="87" customHeight="1">
+      <c r="A36" s="101" t="inlineStr">
         <is>
           <t>DUE : prime pool remplacement — Assistantes Médicales</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="92" t="n"/>
+      <c r="C36" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="102" t="inlineStr">
         <is>
           <t>22/04/2024 (DUE)</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="103" t="inlineStr">
         <is>
           <t>DUE prime pool remplacement assistantes medicales 2024.pdf</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="103" t="inlineStr">
         <is>
           <t>DUE_Prime de Pool de remplacement _ Assistantes Médicales Vfinale.docx</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="103" t="inlineStr">
         <is>
           <t>resume-due-prime-pool-remplacement-am.md</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H36" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_pool_remplacement_FO.pdf</t>
         </is>
       </c>
-      <c r="I36" s="6" t="n">
+      <c r="I36" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="J36" s="103" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
         </is>
       </c>
-      <c r="K36" s="25" t="inlineStr">
+      <c r="K36" s="103" t="inlineStr">
         <is>
           <t>Point 2 : 'd'autre part' sans 'd'une part' correspondant -- construction orpheline. Preambule incoherent : decrit une negociation ratee sur un 'parcours professionnel complementaire' puis bascule sans lien apparent sur la prime de pool de remplacement -- semble etre un texte repris d'un autre dossier sans adaptation.</t>
         </is>
       </c>
-      <c r="L36" s="25" t="inlineStr">
+      <c r="L36" s="103" t="inlineStr">
         <is>
           <t>Aucun mecanisme identifie -- seule une information administrative RH lors de la sortie du pool est prevue (point 4).</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="27" t="inlineStr">
+    <row r="37" ht="46.5" customHeight="1">
+      <c r="A37" s="101" t="inlineStr">
         <is>
           <t>DUE : prime pool remplacement — AS / IDE</t>
         </is>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B37" s="92" t="n"/>
+      <c r="C37" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
+      <c r="D37" s="102" t="inlineStr">
         <is>
           <t>22/04/2024 (DUE)</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E37" s="103" t="inlineStr">
         <is>
           <t>DUE prime pool remplacement AS IDE 2024.pdf</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
+      <c r="F37" s="103" t="inlineStr">
         <is>
           <t>DUE_Prime de Pool de remplacement _ soignants Version Définitive.docx</t>
         </is>
       </c>
-      <c r="G37" s="8" t="inlineStr">
+      <c r="G37" s="103" t="inlineStr">
         <is>
           <t>resume-due-prime-pool-remplacement-soignants.md</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr">
+      <c r="H37" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_prime_pool_remplacement_FO.pdf</t>
         </is>
       </c>
-      <c r="I37" s="10" t="n">
+      <c r="I37" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J37" s="8" t="inlineStr">
+      <c r="J37" s="103" t="inlineStr">
         <is>
           <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
         </is>
       </c>
-      <c r="K37" s="25" t="inlineStr">
+      <c r="K37" s="103" t="inlineStr">
         <is>
           <t>Meme construction orpheline 'd'autre part' sans 'd'une part' (point 2). Preambule coherent avec son objet, contrairement a la version Assistants medicaux.</t>
         </is>
       </c>
-      <c r="L37" s="25" t="inlineStr">
+      <c r="L37" s="103" t="inlineStr">
         <is>
           <t>Aucun mecanisme identifie -- seule l'information administrative des Cadres de Sante vers la RH est prevue (point 4).</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="90" customHeight="1">
-      <c r="A38" s="26" t="inlineStr">
+    <row r="38" ht="73.5" customHeight="1">
+      <c r="A38" s="95" t="inlineStr">
         <is>
           <t>Chèques syndicaux</t>
         </is>
       </c>
-      <c r="B38" s="9" t="inlineStr">
+      <c r="B38" s="92" t="n"/>
+      <c r="C38" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" s="96" t="inlineStr">
         <is>
           <t>03/10/2022</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="97" t="inlineStr">
         <is>
           <t>Accord-Cheques syndicaux_v signee.pdf</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="97" t="inlineStr">
         <is>
           <t>Accord chèques syndicaux_v2022-09-22.docx</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G38" s="97" t="inlineStr">
         <is>
           <t>resume-cheques-syndicaux.md</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H38" s="97" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I38" s="6" t="n">
+      <c r="I38" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J38" s="97" t="inlineStr">
         <is>
           <t>20/10/2026 : doublon avec accent supprimé (PDF « v signée »). Pas de dépliant (hors périmètre dépliant). PDF servi par le site mais non listé (lien sur le Thème).</t>
         </is>
       </c>
-      <c r="K38" s="25" t="inlineStr">
+      <c r="K38" s="97" t="inlineStr">
         <is>
           <t>Audit repris le 20/10/2026 (David confirme n'avoir jamais demande l'arret de la verification). Aucune coquille relevee dans le corps de l'accord (numerotation Articles 1-6 coherente, texte clair).</t>
         </is>
       </c>
-      <c r="L38" s="25" t="inlineStr">
+      <c r="L38" s="97" t="inlineStr">
         <is>
           <t>Revision (Art. 4, modalites du code du travail) ; duree indeterminee, entree en vigueur le lendemain du depot (Art. 5) ; publicite (Art. 6, TeleAccords + greffe CPH Angers). Aucune commission de suivi, bilan ou indicateur specifique prevu.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="27" t="inlineStr">
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2023</t>
         </is>
       </c>
-      <c r="B39" s="13" t="inlineStr">
+      <c r="B39" s="92" t="n"/>
+      <c r="C39" s="108" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
+      <c r="D39" s="108" t="inlineStr">
         <is>
           <t>08/06/2023</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E39" s="109" t="inlineStr">
         <is>
           <t>PV Desaccord NAO 2023.pdf</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="109" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G39" s="8" t="inlineStr">
+      <c r="G39" s="109" t="inlineStr">
         <is>
           <t>PV Desaccord NAO 2023.md</t>
         </is>
       </c>
-      <c r="H39" s="8" t="inlineStr">
+      <c r="H39" s="109" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I39" s="10" t="n">
+      <c r="I39" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="8" t="n"/>
-      <c r="K39" s="25" t="n"/>
-      <c r="L39" s="25" t="n"/>
-    </row>
-    <row r="40" ht="105" customHeight="1">
-      <c r="A40" s="26" t="inlineStr">
+      <c r="J39" s="109" t="n"/>
+      <c r="K39" s="109" t="n"/>
+      <c r="L39" s="109" t="n"/>
+    </row>
+    <row r="40" ht="73.5" customHeight="1">
+      <c r="A40" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2024</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="92" t="n"/>
+      <c r="C40" s="108" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D40" s="108" t="inlineStr">
         <is>
           <t>18/04/2024</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="109" t="inlineStr">
         <is>
           <t>NAO 2024 - PV Désaccord.pdf</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F40" s="109" t="inlineStr">
         <is>
           <t>PV NAO 2024 - V Finale plus en vigueur.docx</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="109" t="inlineStr">
         <is>
           <t>NAO 2024 - PV Desaccord.md</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H40" s="109" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I40" s="6" t="n">
+      <c r="I40" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="J40" s="109" t="inlineStr">
         <is>
           <t>Fichier Word ajouté le 20/10/2026 par David Di Peri. Contenu comparé intégralement au .md existant (lui-même issu du PDF signé) : aucun écart trouvé. Date et signature (Pr Mario Campone, Directeur Général, seul signataire) verifiees visuellement sur le PDF signe le 20/10/2026 : conformes (18/04/2024).</t>
         </is>
       </c>
-      <c r="K40" s="25" t="n"/>
-      <c r="L40" s="25" t="n"/>
-    </row>
-    <row r="41" ht="105" customHeight="1">
-      <c r="A41" s="27" t="inlineStr">
+      <c r="K40" s="109" t="n"/>
+      <c r="L40" s="109" t="n"/>
+    </row>
+    <row r="41" ht="73.5" customHeight="1">
+      <c r="A41" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2025</t>
         </is>
       </c>
-      <c r="B41" s="13" t="inlineStr">
+      <c r="B41" s="92" t="n"/>
+      <c r="C41" s="108" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D41" s="108" t="inlineStr">
         <is>
           <t>13/10/2025</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E41" s="109" t="inlineStr">
         <is>
           <t>NAO 2025 - Procès verbal de désaccord.pdf</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="109" t="inlineStr">
         <is>
           <t>PV NAO 2025 - V 2 plus en vigueur.docx</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr">
+      <c r="G41" s="109" t="inlineStr">
         <is>
           <t>pv-desaccord-nao-2025.md</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="H41" s="109" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I41" s="10" t="n">
+      <c r="I41" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="8" t="inlineStr">
+      <c r="J41" s="109" t="inlineStr">
         <is>
           <t>Fichier Word ajouté le 20/10/2026 par David Di Peri. Contenu comparé intégralement au .md existant (lui-même issu du PDF signé) : aucun écart trouvé. Date et signature (Pr Mario Campone, Directeur Général, seul signataire) verifiees visuellement sur le PDF signe le 20/10/2026 : conformes (13/10/2025).</t>
         </is>
       </c>
-      <c r="K41" s="25" t="n"/>
-      <c r="L41" s="25" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="26" t="inlineStr">
+      <c r="K41" s="109" t="n"/>
+      <c r="L41" s="109" t="n"/>
+    </row>
+    <row r="42" ht="33" customHeight="1">
+      <c r="A42" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2026</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="92" t="n"/>
+      <c r="C42" s="108" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
       </c>
-      <c r="C42" s="13" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" s="108" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E42" s="109" t="inlineStr">
         <is>
           <t>NAO 2026 _PV de désaccord signé.pdf</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F42" s="109" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="G42" s="109" t="inlineStr">
         <is>
           <t>NAO 2026 _PV de desaccord signe.md</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="H42" s="109" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I42" s="6" t="n">
+      <c r="I42" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="4" t="n"/>
-      <c r="K42" s="25" t="n"/>
-      <c r="L42" s="25" t="n"/>
-    </row>
-    <row r="43" ht="105" customHeight="1">
-      <c r="A43" s="27" t="inlineStr">
+      <c r="J42" s="109" t="n"/>
+      <c r="K42" s="109" t="n"/>
+      <c r="L42" s="109" t="n"/>
+    </row>
+    <row r="43" ht="73.5" customHeight="1">
+      <c r="A43" s="91" t="inlineStr">
         <is>
           <t>Grille de rémunération et de classification — personnel non praticien</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="92" t="n"/>
+      <c r="C43" s="93" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D43" s="10" t="inlineStr">
+      <c r="D43" s="93" t="inlineStr">
         <is>
           <t>2025-01-01 (date tirée du nom du fichier)</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E43" s="94" t="inlineStr">
         <is>
           <t>2025-01-01 Grille de rémunération CLCC non praticiens.pdf</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F43" s="94" t="inlineStr">
         <is>
           <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr">
+      <c r="G43" s="94" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="H43" s="8" t="inlineStr">
+      <c r="H43" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I43" s="10" t="n">
+      <c r="I43" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="J43" s="8" t="inlineStr">
+      <c r="J43" s="94" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — corrigée à la date figurant dans le nom du fichier (2025-01-01), à confirmer. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
         </is>
       </c>
-      <c r="K43" s="25" t="n"/>
-      <c r="L43" s="25" t="n"/>
-    </row>
-    <row r="44" ht="105" customHeight="1">
-      <c r="A44" s="26" t="inlineStr">
+      <c r="K43" s="94" t="n"/>
+      <c r="L43" s="94" t="n"/>
+    </row>
+    <row r="44" ht="73.5" customHeight="1">
+      <c r="A44" s="91" t="inlineStr">
         <is>
           <t>Grille de rémunération — praticiens</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B44" s="92" t="n"/>
+      <c r="C44" s="93" t="inlineStr">
         <is>
           <t>CCN</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" s="93" t="inlineStr">
         <is>
           <t>non précisée dans le fichier</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E44" s="94" t="inlineStr">
         <is>
           <t>Grille rémunération praticien.pdf</t>
         </is>
       </c>
-      <c r="F44" s="21" t="inlineStr">
+      <c r="F44" s="94" t="inlineStr">
         <is>
           <t>non applicable (texte de branche FNCLCC/Unicancer, jamais rédigé par l'ICO)</t>
         </is>
       </c>
-      <c r="G44" s="7" t="inlineStr">
+      <c r="G44" s="94" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H44" s="94" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I44" s="6" t="n">
+      <c r="I44" s="93" t="n">
         <v>0</v>
       </c>
-      <c r="J44" s="4" t="inlineStr">
+      <c r="J44" s="94" t="inlineStr">
         <is>
           <t>⚠️ CORRECTION : date affichait 'consolidée au 01/02/2026' (copiée par erreur depuis la ligne CCN texte) — aucune date vérifiée dans le fichier lui-même, laissée non précisée plutôt que d'en inventer une. Confirmé par David (19/10/2026) : pas de Word d'origine, texte/grille de branche — ne jamais chercher.</t>
         </is>
       </c>
-      <c r="K44" s="25" t="n"/>
-      <c r="L44" s="25" t="n"/>
-    </row>
-    <row r="45" ht="135" customHeight="1">
-      <c r="A45" s="27" t="inlineStr">
+      <c r="K44" s="94" t="n"/>
+      <c r="L44" s="94" t="n"/>
+    </row>
+    <row r="45" ht="100.5" customHeight="1">
+      <c r="A45" s="95" t="inlineStr">
         <is>
           <t>Accord intergénérationnel</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="97" t="n"/>
+      <c r="C45" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D45" s="10" t="inlineStr">
+      <c r="D45" s="96" t="inlineStr">
         <is>
           <t>30/01/2020</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="97" t="inlineStr">
         <is>
           <t>Accord Intergénérationnel du 30 01 2020_signé.pdf</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="97" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G45" s="8" t="inlineStr">
+      <c r="G45" s="97" t="inlineStr">
         <is>
           <t>resume-intergenerationnel.md</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="H45" s="97" t="inlineStr">
         <is>
           <t>Depliant_intergenerationnel_FO.pdf</t>
         </is>
       </c>
-      <c r="I45" s="10" t="n">
+      <c r="I45" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="J45" s="97" t="inlineStr">
         <is>
           <t>Corrigé le 20/10/2026 : l'avenant n°1 (30/06/2021) a été restauré au catalogue (voir ligne dédiée), toujours en vigueur en parallèle de l'avenant 2023 (aucun des deux ne s'abroge expressément). Signataires de l'accord de 2020 (lecture du PDF signé) : CGT-FO, Sud et CFE-CGC ; la CFDT n'a pas signé. ⚠️ Point ouvert : date du 30/01/2020 (clause de signature) contre séance du 3 février 2020 (art. 6.5), voir colonne Coquilles.</t>
         </is>
       </c>
-      <c r="K45" s="25" t="inlineStr">
+      <c r="K45" s="97" t="inlineStr">
         <is>
           <t>Contradiction de date : Art. 6.5 indique une signature 'le 3 fevrier 2020', alors que la clause de signature finale indique 'Fait a Angers, le 30 janvier 2020' -- deux dates differentes pour le meme evenement. Saut de numerotation : l'Art. 3.2 a des sous-parties numerotees a tort '3.3.1'/'3.3.2' au lieu de '3.2.1'/'3.2.2'.</t>
         </is>
       </c>
-      <c r="L45" s="25" t="inlineStr">
+      <c r="L45" s="97" t="inlineStr">
         <is>
           <t>Indicateur par objectif (Art. 6.1) ; bilan annuel au CSE central au 2e trimestre + transmission aux OS signataires (6.1) ; clause de revoyure apres la 1ere annee (6.1) ; duree indeterminee (6.2).</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="90" customHeight="1">
-      <c r="A46" s="26" t="inlineStr">
+    <row r="46" ht="154.5" customHeight="1">
+      <c r="A46" s="98" t="n"/>
+      <c r="B46" s="99" t="inlineStr">
+        <is>
+          <t>Avenant - Accord intergenerationnel n1 (30/06/2021)</t>
+        </is>
+      </c>
+      <c r="C46" s="100" t="inlineStr">
+        <is>
+          <t>Accord local</t>
+        </is>
+      </c>
+      <c r="D46" s="100" t="inlineStr">
+        <is>
+          <t>30/06/2021</t>
+        </is>
+      </c>
+      <c r="E46" s="98" t="inlineStr">
+        <is>
+          <t>Accord Intergenerationnel Avenant n1 signe.pdf</t>
+        </is>
+      </c>
+      <c r="F46" s="98" t="inlineStr">
+        <is>
+          <t>Accord Intergénérationnel_Avenant n°1_vDéfinitive plus en vigueur.docx (dossier archive-accords-locaux/Format word ; version de travail définitive avant signature ; le nom du fichier dit « plus en vigueur », à renommer ou à confirmer)</t>
+        </is>
+      </c>
+      <c r="G46" s="98" t="inlineStr">
+        <is>
+          <t>resume-intergenerationnel.md</t>
+        </is>
+      </c>
+      <c r="H46" s="98" t="inlineStr">
+        <is>
+          <t>Depliant_intergenerationnel_FO.pdf</t>
+        </is>
+      </c>
+      <c r="I46" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="98" t="inlineStr">
+        <is>
+          <t>Restaure le 20/10/2026 -- avait ete classe a tort 'plus en vigueur' et archive ; aucun texte posterieur ne l'abroge (regle avenants, David 20/10/2026). Ajoute la possibilite de fractionner un temps partiel a 50% sur 2 semaines (Art. 3.4.2). PDF servi par le site mais non listé (lien sur le Thème).</t>
+        </is>
+      </c>
+      <c r="K46" s="98" t="inlineStr">
+        <is>
+          <t>Section finale non numerotee : intitulee litteralement 'ARTICLE X -- DISPOSITIONS FINALES' (placeholder laisse tel quel), sous-parties 'X.1'/'X.2'. Pas de clause de revision ni de denonciation propre (contrairement a l'accord de base et a l'avenant 2023).</t>
+        </is>
+      </c>
+      <c r="L46" s="98" t="inlineStr">
+        <is>
+          <t>Aucune clause de suivi propre identifiee dans cet avenant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="127.5" customHeight="1">
+      <c r="A47" s="98" t="n"/>
+      <c r="B47" s="99" t="inlineStr">
         <is>
           <t>Avenant — Accord intergénérationnel (15/09/2023)</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="C47" s="100" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="100" t="inlineStr">
         <is>
           <t>15/09/2023</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="98" t="inlineStr">
         <is>
           <t>Avenant accord d'entreprise intergénérationnel_2023_Version signée.pdf</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F47" s="98" t="inlineStr">
         <is>
           <t>Avenant Accord Intergénérationnel 2023 plus en vigueur.docx (dossier archive-accords-locaux/Format word ; le nom du fichier dit « plus en vigueur », à renommer ou à confirmer)</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G47" s="98" t="inlineStr">
         <is>
           <t>resume-intergenerationnel.md</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H47" s="98" t="inlineStr">
         <is>
           <t>Depliant_intergenerationnel_FO.pdf</t>
         </is>
       </c>
-      <c r="I46" s="6" t="n">
+      <c r="I47" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="J46" s="4" t="inlineStr">
+      <c r="J47" s="98" t="inlineStr">
         <is>
           <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Modifie l'art. 3.4.2 (temps partiel fin de carrière). Aucun Word reçu. 20/10/2026 : Word retrouvé dans l'archive (non comparé au PDF signé dans cette passe).</t>
         </is>
       </c>
-      <c r="K46" s="25" t="inlineStr">
+      <c r="K47" s="98" t="inlineStr">
         <is>
           <t>Art. 2.3 (Denonciation) : 'DREET d'Angers' -- lettre 'S' manquante.</t>
         </is>
       </c>
-      <c r="L46" s="25" t="inlineStr">
+      <c r="L47" s="98" t="inlineStr">
         <is>
           <t>Aucune clause de suivi propre a cet avenant (il ne modifie que les conditions d'eligibilite de l'Art. 3.4.2).</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="120" customHeight="1">
-      <c r="A47" s="27" t="inlineStr">
+    <row r="48" ht="87" customHeight="1">
+      <c r="A48" s="95" t="inlineStr">
         <is>
           <t>Plan d'Épargne d'Entreprise (PEE)</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B48" s="92" t="n"/>
+      <c r="C48" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
+      <c r="D48" s="96" t="inlineStr">
         <is>
           <t>22/02/2019</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E48" s="97" t="inlineStr">
         <is>
           <t>Accord PEE signe par FO et CGC.pdf</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F48" s="97" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="G48" s="97" t="inlineStr">
         <is>
           <t>resume_PEE_2019.md (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="H48" s="97" t="inlineStr">
         <is>
           <t>Depliant_PEE_FO.pdf (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="I47" s="10" t="n">
+      <c r="I48" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J47" s="8" t="inlineStr">
+      <c r="J48" s="97" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG le 22/02/2019 — CGT-FO et CFE-CGC signataires, CGT et Sud Santé-Sociaux non signataires. 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Accord PEE signe par FO et CGC.md ». ⚠️ À vérifier : abondement du PEE.</t>
         </is>
       </c>
-      <c r="K47" s="25" t="n"/>
-      <c r="L47" s="25" t="n"/>
-    </row>
-    <row r="48" ht="150" customHeight="1">
-      <c r="A48" s="26" t="inlineStr">
+      <c r="K48" s="97" t="n"/>
+      <c r="L48" s="97" t="n"/>
+    </row>
+    <row r="49" ht="100.5" customHeight="1">
+      <c r="A49" s="97" t="n"/>
+      <c r="B49" s="95" t="inlineStr">
         <is>
           <t>Avenant — Indemnité de restauration</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="C49" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="96" t="inlineStr">
         <is>
           <t>15/11/2016</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="97" t="inlineStr">
         <is>
           <t>Avenant indemnite restauration 2016.pdf</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F49" s="97" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G49" s="97" t="inlineStr">
         <is>
           <t>resume_avenant_indemnite_restauration_2016.md (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr">
+      <c r="H49" s="97" t="inlineStr">
         <is>
           <t>Depliant_avenant_indemnite_restauration_FO.pdf (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="I48" s="6" t="n">
+      <c r="I49" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J48" s="4" t="inlineStr">
+      <c r="J49" s="97" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Avenant n°1 à l'accord du 19/12/2013 (accord de base non retrouvé). Signé par le DG et les 4 OS. 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Avenant indemnite restauration 2016.md ». ⚠️ À vérifier : le montant de l'indemnité ne figure pas dans l'avenant (accord de base du 19/12/2013 non retrouvé).</t>
         </is>
       </c>
-      <c r="K48" s="25" t="n"/>
-      <c r="L48" s="25" t="n"/>
-    </row>
-    <row r="49" ht="135" customHeight="1">
-      <c r="A49" s="27" t="inlineStr">
+      <c r="K49" s="97" t="n"/>
+      <c r="L49" s="97" t="n"/>
+    </row>
+    <row r="50" ht="100.5" customHeight="1">
+      <c r="A50" s="95" t="inlineStr">
         <is>
           <t>Don de jours de repos non pris</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B50" s="92" t="n"/>
+      <c r="C50" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="D50" s="96" t="inlineStr">
         <is>
           <t>09/01/2015</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E50" s="97" t="inlineStr">
         <is>
           <t>Accord don de jours de repos 2015.pdf</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F50" s="97" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G50" s="97" t="inlineStr">
         <is>
           <t>resume_don_jours_repos_2015.md (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="H50" s="97" t="inlineStr">
         <is>
           <t>Depliant_don_jours_repos_FO.pdf (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="I49" s="10" t="n">
+      <c r="I50" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J49" s="8" t="inlineStr">
+      <c r="J50" s="97" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG et les 4 OS. En-tête du PDF porte une date de projet non mise à jour (sans incidence). 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Accord don de jours de repos 2015.md ». ⚠️ À vérifier : l'en-tête du PDF porte la mention « Projet accord ».</t>
         </is>
       </c>
-      <c r="K49" s="25" t="n"/>
-      <c r="L49" s="25" t="n"/>
-    </row>
-    <row r="50" ht="120" customHeight="1">
-      <c r="A50" s="26" t="inlineStr">
+      <c r="K50" s="97" t="n"/>
+      <c r="L50" s="97" t="n"/>
+    </row>
+    <row r="51" ht="87" customHeight="1">
+      <c r="A51" s="101" t="inlineStr">
         <is>
           <t>Charte unilatérale sur le droit à la déconnexion</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
+      <c r="B51" s="92" t="n"/>
+      <c r="C51" s="102" t="inlineStr">
         <is>
           <t>DUE</t>
         </is>
       </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D51" s="102" t="inlineStr">
         <is>
           <t>22/06/2018 (DUE)</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E51" s="103" t="inlineStr">
         <is>
           <t>Charte deconnexion 2018.pdf</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
+      <c r="F51" s="103" t="inlineStr">
         <is>
           <t>manquant</t>
         </is>
       </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="G51" s="103" t="inlineStr">
         <is>
           <t>resume_charte_deconnexion_2018.md (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H51" s="103" t="inlineStr">
         <is>
           <t>Depliant_DUE_deconnexion_FO.pdf (dossier en_attente_version_word)</t>
         </is>
       </c>
-      <c r="I50" s="6" t="n">
+      <c r="I51" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J50" s="4" t="inlineStr">
+      <c r="J51" s="103" t="inlineStr">
         <is>
           <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). DUE (pas un accord négocié) : seule la CFE-CGC avait signé l'accord proposé, négociation non aboutie. Signée par le DG seul. 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Charte deconnexion 2018.md ».</t>
         </is>
       </c>
-      <c r="K50" s="25" t="n"/>
-      <c r="L50" s="25" t="n"/>
-    </row>
-    <row r="51" ht="120" customHeight="1">
-      <c r="A51" s="28" t="inlineStr">
-        <is>
-          <t>Avenant - Accord intergenerationnel n1 (30/06/2021)</t>
-        </is>
-      </c>
-      <c r="B51" s="25" t="inlineStr">
+      <c r="K51" s="103" t="n"/>
+      <c r="L51" s="103" t="n"/>
+    </row>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="95" t="inlineStr">
+        <is>
+          <t>Accord de methode NAO 2026</t>
+        </is>
+      </c>
+      <c r="B52" s="92" t="n"/>
+      <c r="C52" s="96" t="inlineStr">
         <is>
           <t>Accord local</t>
         </is>
       </c>
-      <c r="C51" s="25" t="inlineStr">
-        <is>
-          <t>Avenant</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="inlineStr">
-        <is>
-          <t>30/06/2021</t>
-        </is>
-      </c>
-      <c r="E51" s="25" t="inlineStr">
-        <is>
-          <t>Accord Intergenerationnel Avenant n1 signe.pdf</t>
-        </is>
-      </c>
-      <c r="F51" s="25" t="inlineStr">
-        <is>
-          <t>Accord Intergénérationnel_Avenant n°1_vDéfinitive plus en vigueur.docx (dossier archive-accords-locaux/Format word ; version de travail définitive avant signature ; le nom du fichier dit « plus en vigueur », à renommer ou à confirmer)</t>
-        </is>
-      </c>
-      <c r="G51" s="25" t="inlineStr">
-        <is>
-          <t>resume-intergenerationnel.md</t>
-        </is>
-      </c>
-      <c r="H51" s="25" t="inlineStr">
-        <is>
-          <t>Depliant_intergenerationnel_FO.pdf</t>
-        </is>
-      </c>
-      <c r="I51" s="25" t="n">
+      <c r="D52" s="96" t="inlineStr">
+        <is>
+          <t>22/01/2026</t>
+        </is>
+      </c>
+      <c r="E52" s="97" t="inlineStr">
+        <is>
+          <t>Accord de méthode NAO au titre de 2026.pdf</t>
+        </is>
+      </c>
+      <c r="F52" s="97" t="inlineStr">
+        <is>
+          <t>Accord de méthode NAO 2026.docx (dossier nao/NAO Format Word)</t>
+        </is>
+      </c>
+      <c r="G52" s="97" t="inlineStr">
+        <is>
+          <t>resume-methode-nao-2026.md</t>
+        </is>
+      </c>
+      <c r="H52" s="97" t="inlineStr">
+        <is>
+          <t>-- (aucun, hors format depliant)</t>
+        </is>
+      </c>
+      <c r="I52" s="96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="97" t="inlineStr">
+        <is>
+          <t>Ligne ajoutee le 20/10/2026 (absente du tableau jusqu'ici). 20/10/2026 : PDF signé et Word retrouvés dans le dépôt (la ligne les indiquait manquants). PDF servi par le site mais non listé (lien sur le Thème).</t>
+        </is>
+      </c>
+      <c r="K52" s="97" t="inlineStr">
+        <is>
+          <t>Art. 5.3 : 'DREET d'Angers' -- lettre 'S' manquante. Dates des 3 reunions verifiees par calcul calendaire, toutes correctes.</t>
+        </is>
+      </c>
+      <c r="L52" s="97" t="inlineStr">
+        <is>
+          <t>Compte rendu ecrit sous 5 jours apres chaque reunion, PV final a l'automne 2026 (Art. 4.1/4.3) ; duree determinee, fin a l'issue de la NAO 2026 (5.1) ; revision (5.2) ; denonciation (5.3) ; depot (5.4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="195" customHeight="1">
+      <c r="A53" s="110" t="inlineStr">
+        <is>
+          <t>Règlement intérieur de l'ICO</t>
+        </is>
+      </c>
+      <c r="B53" s="92" t="n"/>
+      <c r="C53" s="111" t="inlineStr">
+        <is>
+          <t>Règlement intérieur</t>
+        </is>
+      </c>
+      <c r="D53" s="111" t="inlineStr">
+        <is>
+          <t>Avis CSE Central 02/04/2024, signé 05/04/2024, en vigueur 23/10/2024</t>
+        </is>
+      </c>
+      <c r="E53" s="112" t="inlineStr">
+        <is>
+          <t>Reglement interieur ICO 2024.pdf</t>
+        </is>
+      </c>
+      <c r="F53" s="112" t="inlineStr">
+        <is>
+          <t>manquant</t>
+        </is>
+      </c>
+      <c r="G53" s="112" t="inlineStr">
+        <is>
+          <t>N/A (texte integral uniquement, comme la CCN - pas de resume salarie prevu a ce stade)</t>
+        </is>
+      </c>
+      <c r="H53" s="112" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I53" s="111" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="112" t="inlineStr">
+        <is>
+          <t>Nouveau le 20/10/2026 (David a ajouté le PDF dans le dossier CCN local). Document unilatéral de la Direction (pas un accord négocié, aucune signature syndicale), soumis à l'avis du CSE Central le 02/04/2024. Fichier source récupéré sous un nom de téléchargement Chrome interrompu (« Non confirmé 237163.crdownload ») ; lu et vérifié intégralement (texte extrait + rendu visuel page par page) : les 29 pages sont complètes et cohérentes malgré ce nom de fichier anormal — David a validé la poursuite avec ce fichier après signalement. Converti en .md fidèlement, sans ajout ni omission de contenu. L'Annexe 1 (Charte d'accès et d'usage du système d'information), annoncée en fin de sommaire et de nouveau juste après la signature, n'a PAS de contenu dans ce PDF — seule la page de coordonnées de l'ICO suit la signature. À demander à la DRH. Pas encore de résumé salarié ni de dépliant pour ce document (non prévu dans la demande initiale).</t>
+        </is>
+      </c>
+      <c r="K53" s="112" t="inlineStr">
+        <is>
+          <t>Clause 2.3.4.4 (test salivaire de depistage de drogues) : la phrase du PDF signe contient, sans ponctuation la detachant du reste, l incise « si elle le souhaite ajouter le cas echeant « et d un salarie assistant l employeur » » qui ressemble a une note de redaction/modele non retiree avant signature (verifie visuellement page 22). Reproduite mot pour mot dans le .md, sans crochets ajoutes ; probablement une erreur de mise en forme cote Direction a signaler.</t>
+        </is>
+      </c>
+      <c r="L53" s="112" t="inlineStr">
+        <is>
+          <t>Aucune clause de bilan, de révision périodique ou de commission de suivi identifiée dans le texte : la seule procédure de modification prévue (art. 4.2) est la reprise de la procédure légale complète (avis du CSE Central) en cas de changement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="73.5" customHeight="1">
+      <c r="A54" s="101" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance (en realite frais de sante) 2022 - Non cadre</t>
+        </is>
+      </c>
+      <c r="B54" s="92" t="n"/>
+      <c r="C54" s="102" t="inlineStr">
+        <is>
+          <t>DUE</t>
+        </is>
+      </c>
+      <c r="D54" s="102" t="inlineStr">
+        <is>
+          <t>25/04/2022 (DUE)</t>
+        </is>
+      </c>
+      <c r="E54" s="103" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance 2022 Non cadre ICO.pdf</t>
+        </is>
+      </c>
+      <c r="F54" s="103" t="n"/>
+      <c r="G54" s="103" t="inlineStr">
+        <is>
+          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
+        </is>
+      </c>
+      <c r="H54" s="103" t="n"/>
+      <c r="I54" s="102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="103" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes).</t>
+        </is>
+      </c>
+      <c r="K54" s="103" t="inlineStr">
+        <is>
+          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
+        </is>
+      </c>
+      <c r="L54" s="103" t="inlineStr">
+        <is>
+          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="100.5" customHeight="1">
+      <c r="A55" s="101" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance (en realite frais de sante) 2022 - Cadre</t>
+        </is>
+      </c>
+      <c r="B55" s="92" t="n"/>
+      <c r="C55" s="102" t="inlineStr">
+        <is>
+          <t>DUE</t>
+        </is>
+      </c>
+      <c r="D55" s="102" t="inlineStr">
+        <is>
+          <t>25/04/2022 (DUE)</t>
+        </is>
+      </c>
+      <c r="E55" s="103" t="inlineStr">
+        <is>
+          <t>DUE Prevoyance 2022 Cadre ICO.pdf</t>
+        </is>
+      </c>
+      <c r="F55" s="103" t="n"/>
+      <c r="G55" s="103" t="inlineStr">
+        <is>
+          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
+        </is>
+      </c>
+      <c r="H55" s="103" t="n"/>
+      <c r="I55" s="102" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="103" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Difference avec la version non cadre : perimetre (positions 6-7 CCN + praticiens) et cotisations (3 tranches PASS au lieu de 2, taux differents).</t>
+        </is>
+      </c>
+      <c r="K55" s="103" t="inlineStr">
+        <is>
+          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
+        </is>
+      </c>
+      <c r="L55" s="103" t="inlineStr">
+        <is>
+          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="73.5" customHeight="1">
+      <c r="A56" s="113" t="inlineStr">
+        <is>
+          <t>Prevoyance AXA (deces, incapacite, invalidite) - Non cadre</t>
+        </is>
+      </c>
+      <c r="B56" s="92" t="n"/>
+      <c r="C56" s="114" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="D56" s="114" t="inlineStr">
+        <is>
+          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
+        </is>
+      </c>
+      <c r="E56" s="115" t="inlineStr">
+        <is>
+          <t>Notice prevoyance non cadres AXA 2015.pdf</t>
+        </is>
+      </c>
+      <c r="F56" s="115" t="n"/>
+      <c r="G56" s="115" t="inlineStr">
+        <is>
+          <t>resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="H56" s="115" t="inlineStr">
+        <is>
+          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
+        </is>
+      </c>
+      <c r="I56" s="114" t="n">
         <v>1</v>
       </c>
-      <c r="J51" s="25" t="inlineStr">
-        <is>
-          <t>Restaure le 20/10/2026 -- avait ete classe a tort 'plus en vigueur' et archive ; aucun texte posterieur ne l'abroge (regle avenants, David 20/10/2026). Ajoute la possibilite de fractionner un temps partiel a 50% sur 2 semaines (Art. 3.4.2). PDF servi par le site mais non listé (lien sur le Thème).</t>
-        </is>
-      </c>
-      <c r="K51" s="25" t="inlineStr">
-        <is>
-          <t>Section finale non numerotee : intitulee litteralement 'ARTICLE X -- DISPOSITIONS FINALES' (placeholder laisse tel quel), sous-parties 'X.1'/'X.2'. Pas de clause de revision ni de denonciation propre (contrairement a l'accord de base et a l'avenant 2023).</t>
-        </is>
-      </c>
-      <c r="L51" s="25" t="inlineStr">
-        <is>
-          <t>Aucune clause de suivi propre identifiee dans cet avenant.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="90" customHeight="1">
-      <c r="A52" s="28" t="inlineStr">
-        <is>
-          <t>Accord de methode NAO 2026</t>
-        </is>
-      </c>
-      <c r="B52" s="25" t="inlineStr">
-        <is>
-          <t>Accord local</t>
-        </is>
-      </c>
-      <c r="C52" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D52" s="25" t="inlineStr">
-        <is>
-          <t>22/01/2026</t>
-        </is>
-      </c>
-      <c r="E52" s="25" t="inlineStr">
-        <is>
-          <t>Accord de méthode NAO au titre de 2026.pdf</t>
-        </is>
-      </c>
-      <c r="F52" s="25" t="inlineStr">
-        <is>
-          <t>Accord de méthode NAO 2026.docx (dossier nao/NAO Format Word)</t>
-        </is>
-      </c>
-      <c r="G52" s="25" t="inlineStr">
-        <is>
-          <t>resume-methode-nao-2026.md</t>
-        </is>
-      </c>
-      <c r="H52" s="25" t="inlineStr">
-        <is>
-          <t>-- (aucun, hors format depliant)</t>
-        </is>
-      </c>
-      <c r="I52" s="25" t="n">
+      <c r="J56" s="115" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604120000Q. Garanties verifiees identiques mot pour mot a la version cadre (comparaison textuelle programmatique page par page) -- seul le perimetre des beneficiaires et le numero de contrat different. Resume unique cadre+non cadre avec clause beneficiaire integree.</t>
+        </is>
+      </c>
+      <c r="K56" s="115" t="n"/>
+      <c r="L56" s="115" t="inlineStr">
+        <is>
+          <t>Information individuelle (notice remise a chaque salarie, Art. 9) ; portabilite en cas de rupture ouvrant droit au chomage (maintien loi 2013) ; maintien des garanties deces au profit des beneficiaires de rentes en cas de changement d'organisme assureur (Art. 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1">
+      <c r="A57" s="113" t="inlineStr">
+        <is>
+          <t>Prevoyance AXA (deces, incapacite, invalidite) - Cadre</t>
+        </is>
+      </c>
+      <c r="B57" s="92" t="n"/>
+      <c r="C57" s="114" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="D57" s="114" t="inlineStr">
+        <is>
+          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
+        </is>
+      </c>
+      <c r="E57" s="115" t="inlineStr">
+        <is>
+          <t>Notice prevoyance cadres AXA 2015.pdf</t>
+        </is>
+      </c>
+      <c r="F57" s="115" t="n"/>
+      <c r="G57" s="115" t="inlineStr">
+        <is>
+          <t>resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="H57" s="115" t="inlineStr">
+        <is>
+          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
+        </is>
+      </c>
+      <c r="I57" s="114" t="n">
         <v>0</v>
       </c>
-      <c r="J52" s="25" t="inlineStr">
-        <is>
-          <t>Ligne ajoutee le 20/10/2026 (absente du tableau jusqu'ici). 20/10/2026 : PDF signé et Word retrouvés dans le dépôt (la ligne les indiquait manquants). PDF servi par le site mais non listé (lien sur le Thème).</t>
-        </is>
-      </c>
-      <c r="K52" s="25" t="inlineStr">
-        <is>
-          <t>Art. 5.3 : 'DREET d'Angers' -- lettre 'S' manquante. Dates des 3 reunions verifiees par calcul calendaire, toutes correctes.</t>
-        </is>
-      </c>
-      <c r="L52" s="25" t="inlineStr">
-        <is>
-          <t>Compte rendu ecrit sous 5 jours apres chaque reunion, PV final a l'automne 2026 (Art. 4.1/4.3) ; duree determinee, fin a l'issue de la NAO 2026 (5.1) ; revision (5.2) ; denonciation (5.3) ; depot (5.4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="300" customHeight="1">
-      <c r="A53" s="28" t="inlineStr">
-        <is>
-          <t>Règlement intérieur de l'ICO</t>
-        </is>
-      </c>
-      <c r="B53" s="25" t="inlineStr">
-        <is>
-          <t>Règlement intérieur</t>
-        </is>
-      </c>
-      <c r="C53" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D53" s="25" t="inlineStr">
-        <is>
-          <t>Avis CSE Central 02/04/2024, signé 05/04/2024, en vigueur 23/10/2024</t>
-        </is>
-      </c>
-      <c r="E53" s="25" t="inlineStr">
-        <is>
-          <t>Reglement interieur ICO 2024.pdf</t>
-        </is>
-      </c>
-      <c r="F53" s="25" t="inlineStr">
-        <is>
-          <t>manquant</t>
-        </is>
-      </c>
-      <c r="G53" s="25" t="inlineStr">
-        <is>
-          <t>N/A (texte integral uniquement, comme la CCN - pas de resume salarie prevu a ce stade)</t>
-        </is>
-      </c>
-      <c r="H53" s="25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I53" s="25" t="n">
+      <c r="J57" s="115" t="inlineStr">
+        <is>
+          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604110000Q. Garanties identiques a la version non cadre (voir ligne ci-dessus) -- meme resume et depliant, compte comme un seul depliant au total (Nb depliants=0 ici pour ne pas compter en double).</t>
+        </is>
+      </c>
+      <c r="K57" s="115" t="n"/>
+      <c r="L57" s="115" t="inlineStr">
+        <is>
+          <t>Identique a la ligne non cadre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="46.5" customHeight="1">
+      <c r="A58" s="113" t="inlineStr">
+        <is>
+          <t>Clause beneficiaire Prevoyance AXA (formulaire)</t>
+        </is>
+      </c>
+      <c r="B58" s="92" t="n"/>
+      <c r="C58" s="114" t="inlineStr">
+        <is>
+          <t>Prevoyance, mutuelle, retraite</t>
+        </is>
+      </c>
+      <c r="D58" s="114" t="inlineStr">
+        <is>
+          <t>VF 2019</t>
+        </is>
+      </c>
+      <c r="E58" s="115" t="inlineStr">
+        <is>
+          <t>Clause beneficiaire Prevoyance AXA 2019.pdf</t>
+        </is>
+      </c>
+      <c r="F58" s="115" t="n"/>
+      <c r="G58" s="115" t="inlineStr">
+        <is>
+          <t>Integree dans resume-prevoyance-axa.md</t>
+        </is>
+      </c>
+      <c r="H58" s="115" t="n"/>
+      <c r="I58" s="114" t="n">
         <v>0</v>
       </c>
-      <c r="J53" s="25" t="inlineStr">
-        <is>
-          <t>Nouveau le 20/10/2026 (David a ajouté le PDF dans le dossier CCN local). Document unilatéral de la Direction (pas un accord négocié, aucune signature syndicale), soumis à l'avis du CSE Central le 02/04/2024. Fichier source récupéré sous un nom de téléchargement Chrome interrompu (« Non confirmé 237163.crdownload ») ; lu et vérifié intégralement (texte extrait + rendu visuel page par page) : les 29 pages sont complètes et cohérentes malgré ce nom de fichier anormal — David a validé la poursuite avec ce fichier après signalement. Converti en .md fidèlement, sans ajout ni omission de contenu. L'Annexe 1 (Charte d'accès et d'usage du système d'information), annoncée en fin de sommaire et de nouveau juste après la signature, n'a PAS de contenu dans ce PDF — seule la page de coordonnées de l'ICO suit la signature. À demander à la DRH. Pas encore de résumé salarié ni de dépliant pour ce document (non prévu dans la demande initiale).</t>
-        </is>
-      </c>
-      <c r="K53" s="25" t="inlineStr">
-        <is>
-          <t>Clause 2.3.4.4 (test salivaire de depistage de drogues) : la phrase du PDF signe contient, sans ponctuation la detachant du reste, l incise « si elle le souhaite ajouter le cas echeant « et d un salarie assistant l employeur » » qui ressemble a une note de redaction/modele non retiree avant signature (verifie visuellement page 22). Reproduite mot pour mot dans le .md, sans crochets ajoutes ; probablement une erreur de mise en forme cote Direction a signaler.</t>
-        </is>
-      </c>
-      <c r="L53" s="25" t="inlineStr">
-        <is>
-          <t>Aucune clause de bilan, de révision périodique ou de commission de suivi identifiée dans le texte : la seule procédure de modification prévue (art. 4.2) est la reprise de la procédure légale complète (avis du CSE Central) en cas de changement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="105" customHeight="1">
-      <c r="A54" s="28" t="inlineStr">
-        <is>
-          <t>DUE Prevoyance (en realite frais de sante) 2022 - Non cadre</t>
-        </is>
-      </c>
-      <c r="B54" s="25" t="inlineStr">
-        <is>
-          <t>DUE</t>
-        </is>
-      </c>
-      <c r="C54" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D54" s="25" t="inlineStr">
-        <is>
-          <t>25/04/2022 (DUE)</t>
-        </is>
-      </c>
-      <c r="E54" s="25" t="inlineStr">
-        <is>
-          <t>DUE Prevoyance 2022 Non cadre ICO.pdf</t>
-        </is>
-      </c>
-      <c r="F54" s="25" t="n"/>
-      <c r="G54" s="25" t="inlineStr">
-        <is>
-          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
-        </is>
-      </c>
-      <c r="H54" s="25" t="n"/>
-      <c r="I54" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="25" t="inlineStr">
-        <is>
-          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes).</t>
-        </is>
-      </c>
-      <c r="K54" s="25" t="inlineStr">
-        <is>
-          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
-        </is>
-      </c>
-      <c r="L54" s="25" t="inlineStr">
-        <is>
-          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="135" customHeight="1">
-      <c r="A55" s="28" t="inlineStr">
-        <is>
-          <t>DUE Prevoyance (en realite frais de sante) 2022 - Cadre</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="inlineStr">
-        <is>
-          <t>DUE</t>
-        </is>
-      </c>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D55" s="25" t="inlineStr">
-        <is>
-          <t>25/04/2022 (DUE)</t>
-        </is>
-      </c>
-      <c r="E55" s="25" t="inlineStr">
-        <is>
-          <t>DUE Prevoyance 2022 Cadre ICO.pdf</t>
-        </is>
-      </c>
-      <c r="F55" s="25" t="n"/>
-      <c r="G55" s="25" t="inlineStr">
-        <is>
-          <t>N/A (document historique, voir resume du regime actuel : resume-due-complementaire-frais-sante.md)</t>
-        </is>
-      </c>
-      <c r="H55" s="25" t="n"/>
-      <c r="I55" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="25" t="inlineStr">
-        <is>
-          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Difference avec la version non cadre : perimetre (positions 6-7 CCN + praticiens) et cotisations (3 tranches PASS au lieu de 2, taux differents).</t>
-        </is>
-      </c>
-      <c r="K55" s="25" t="inlineStr">
-        <is>
-          <t>Titre du document dit 'regime de PREVOYANCE' mais le contenu integral (art. 1 a 11) traite du remboursement des FRAIS DE SANTE, identique dans sa formulation a la DUE 2024 correctement titree. Tres probable erreur de denomination -- David se renseigne aupres de la Direction.</t>
-        </is>
-      </c>
-      <c r="L55" s="25" t="inlineStr">
-        <is>
-          <t>Notice d'information remise a chaque salarie (Art. 9) ; information-consultation du CSE prealable (Art. 10) ; duree indeterminee, modification/denonciation selon la procedure des engagements unilateraux (Art. 11).</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="105" customHeight="1">
-      <c r="A56" s="28" t="inlineStr">
-        <is>
-          <t>Prevoyance AXA (deces, incapacite, invalidite) - Non cadre</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="inlineStr">
+      <c r="J58" s="115" t="inlineStr">
+        <is>
+          <t>Formulaire individuel AXA (reference 480299 04 2017), pas un document contractuel. Contenu integre a la section Clause beneficiaire du resume Prevoyance AXA.</t>
+        </is>
+      </c>
+      <c r="K58" s="115" t="n"/>
+      <c r="L58" s="115" t="n"/>
+    </row>
+    <row r="59" ht="168" customHeight="1">
+      <c r="A59" s="116" t="inlineStr">
+        <is>
+          <t>ICO Information Assistance AXA</t>
+        </is>
+      </c>
+      <c r="B59" s="117" t="n"/>
+      <c r="C59" s="118" t="inlineStr">
         <is>
           <t>Prevoyance, mutuelle, retraite</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D56" s="25" t="inlineStr">
-        <is>
-          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
-        </is>
-      </c>
-      <c r="E56" s="25" t="inlineStr">
-        <is>
-          <t>Notice prevoyance non cadres AXA 2015.pdf</t>
-        </is>
-      </c>
-      <c r="F56" s="25" t="n"/>
-      <c r="G56" s="25" t="inlineStr">
-        <is>
-          <t>resume-prevoyance-axa.md</t>
-        </is>
-      </c>
-      <c r="H56" s="25" t="inlineStr">
-        <is>
-          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
-        </is>
-      </c>
-      <c r="I56" s="25" t="n">
+      <c r="D59" s="118" t="n"/>
+      <c r="E59" s="119" t="inlineStr">
+        <is>
+          <t>ICO Information Assistance AXA.pdf</t>
+        </is>
+      </c>
+      <c r="F59" s="119" t="n"/>
+      <c r="G59" s="119" t="inlineStr">
+        <is>
+          <t>resume-assistance-axa.md (20/10/2026)</t>
+        </is>
+      </c>
+      <c r="H59" s="119" t="inlineStr">
+        <is>
+          <t>Depliant_Assistances_AXA_FO.pdf (20/10/2026)</t>
+        </is>
+      </c>
+      <c r="I59" s="118" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="25" t="inlineStr">
-        <is>
-          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604120000Q. Garanties verifiees identiques mot pour mot a la version cadre (comparaison textuelle programmatique page par page) -- seul le perimetre des beneficiaires et le numero de contrat different. Resume unique cadre+non cadre avec clause beneficiaire integree.</t>
-        </is>
-      </c>
-      <c r="K56" s="25" t="n"/>
-      <c r="L56" s="25" t="inlineStr">
-        <is>
-          <t>Information individuelle (notice remise a chaque salarie, Art. 9) ; portabilite en cas de rupture ouvrant droit au chomage (maintien loi 2013) ; maintien des garanties deces au profit des beneficiaires de rentes en cas de changement d'organisme assureur (Art. 8).</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="90" customHeight="1">
-      <c r="A57" s="28" t="inlineStr">
-        <is>
-          <t>Prevoyance AXA (deces, incapacite, invalidite) - Cadre</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="inlineStr">
-        <is>
-          <t>Prevoyance, mutuelle, retraite</t>
-        </is>
-      </c>
-      <c r="C57" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D57" s="25" t="inlineStr">
-        <is>
-          <t>23/11/2015 (notice AXA, effet 01/01/2016)</t>
-        </is>
-      </c>
-      <c r="E57" s="25" t="inlineStr">
-        <is>
-          <t>Notice prevoyance cadres AXA 2015.pdf</t>
-        </is>
-      </c>
-      <c r="F57" s="25" t="n"/>
-      <c r="G57" s="25" t="inlineStr">
-        <is>
-          <t>resume-prevoyance-axa.md</t>
-        </is>
-      </c>
-      <c r="H57" s="25" t="inlineStr">
-        <is>
-          <t>Depliant_Prevoyance_AXA_FO.pdf</t>
-        </is>
-      </c>
-      <c r="I57" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" s="25" t="inlineStr">
-        <is>
-          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604110000Q. Garanties identiques a la version non cadre (voir ligne ci-dessus) -- meme resume et depliant, compte comme un seul depliant au total (Nb depliants=0 ici pour ne pas compter en double).</t>
-        </is>
-      </c>
-      <c r="K57" s="25" t="n"/>
-      <c r="L57" s="25" t="inlineStr">
-        <is>
-          <t>Identique a la ligne non cadre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="60" customHeight="1">
-      <c r="A58" s="28" t="inlineStr">
-        <is>
-          <t>Clause beneficiaire Prevoyance AXA (formulaire)</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="inlineStr">
-        <is>
-          <t>Prevoyance, mutuelle, retraite</t>
-        </is>
-      </c>
-      <c r="C58" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D58" s="25" t="inlineStr">
-        <is>
-          <t>VF 2019</t>
-        </is>
-      </c>
-      <c r="E58" s="25" t="inlineStr">
-        <is>
-          <t>Clause beneficiaire Prevoyance AXA 2019.pdf</t>
-        </is>
-      </c>
-      <c r="F58" s="25" t="n"/>
-      <c r="G58" s="25" t="inlineStr">
-        <is>
-          <t>Integree dans resume-prevoyance-axa.md</t>
-        </is>
-      </c>
-      <c r="H58" s="25" t="n"/>
-      <c r="I58" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="25" t="inlineStr">
-        <is>
-          <t>Formulaire individuel AXA (reference 480299 04 2017), pas un document contractuel. Contenu integre a la section Clause beneficiaire du resume Prevoyance AXA.</t>
-        </is>
-      </c>
-      <c r="K58" s="25" t="n"/>
-      <c r="L58" s="25" t="n"/>
-    </row>
-    <row r="59" ht="255" customHeight="1">
-      <c r="A59" s="28" t="inlineStr">
-        <is>
-          <t>ICO Information Assistance AXA</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="inlineStr">
-        <is>
-          <t>Prevoyance, mutuelle, retraite</t>
-        </is>
-      </c>
-      <c r="C59" s="25" t="inlineStr">
-        <is>
-          <t>Accord</t>
-        </is>
-      </c>
-      <c r="D59" s="25" t="n"/>
-      <c r="E59" s="25" t="inlineStr">
-        <is>
-          <t>ICO Information Assistance AXA.pdf</t>
-        </is>
-      </c>
-      <c r="F59" s="25" t="n"/>
-      <c r="G59" s="25" t="inlineStr">
-        <is>
-          <t>resume-assistance-axa.md (20/10/2026)</t>
-        </is>
-      </c>
-      <c r="H59" s="25" t="inlineStr">
-        <is>
-          <t>Depliant_Assistances_AXA_FO.pdf (20/10/2026)</t>
-        </is>
-      </c>
-      <c r="I59" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J59" s="25" t="inlineStr">
+      <c r="J59" s="119" t="inlineStr">
         <is>
           <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer. Resume redige et integre le 20/10/2026 sur demande de David : notice d'information des assistances AXA possibles. Erreur corrigee dans le .md source : la condition "aucun membre de la famille a moins de 50 km" ne vise que la presence d'un proche au chevet.</t>
         </is>
       </c>
-      <c r="K59" s="25" t="n"/>
-      <c r="L59" s="25" t="n"/>
+      <c r="K59" s="119" t="n"/>
+      <c r="L59" s="119" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L59"/>
@@ -3946,27 +4080,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId27"/>
@@ -3987,10 +4121,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId51"/>
@@ -4003,6 +4137,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId58"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PV de desaccord NAO 2026 relu en entier, suivi Excel mis a jour
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01THGRE666FhaEFzWEGaAzCH
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -2322,7 +2322,7 @@
       </c>
       <c r="F25" s="98" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G25" s="98" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="J25" s="98" t="inlineStr">
         <is>
-          <t>Ligne créée le 19/10/2026. Aucun Word reçu. Transcription Markdown ajoutée le 20/10/2026 (« AVENANT ACCORD PRIME USC_Version signee.md », relue visuellement contre le PDF). Contenu intégré au résumé et au dépliant : art. 1 (règle d'au moins 50 % de nuits pour les IDE et AS de nuit de Saint-Herblain), art. 2 (règle future après ouverture d'Ambicion / USIP). ⚠️ Point à trancher par David : lecture de la formule applicable après l'ouverture d'Ambicion / USIP (le texte renvoie aux collègues de jour ou d'Angers).</t>
+          <t>Ligne créée le 19/10/2026. Aucun Word reçu. Transcription Markdown ajoutée le 20/10/2026 (« AVENANT ACCORD PRIME USC_Version signee.md », relue visuellement contre le PDF). Contenu intégré au résumé et au dépliant : art. 1 (règle d'au moins 50 % de nuits pour les IDE et AS de nuit de Saint-Herblain), art. 2 (règle future après ouverture d'Ambicion / USIP). ⚠️ Point à trancher par David : lecture de la formule applicable après l'ouverture d'Ambicion / USIP (le texte renvoie aux collègues de jour ou d'Angers). 21/10/2026 : Word toujours en attente de réception.</t>
         </is>
       </c>
       <c r="K25" s="98" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="F39" s="109" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G39" s="109" t="inlineStr">
@@ -3090,7 +3090,11 @@
       <c r="I39" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="109" t="n"/>
+      <c r="J39" s="109" t="inlineStr">
+        <is>
+          <t>Word en attente de réception (David le recherche).</t>
+        </is>
+      </c>
       <c r="K39" s="109" t="n"/>
       <c r="L39" s="109" t="n"/>
     </row>
@@ -3204,7 +3208,7 @@
       </c>
       <c r="D42" s="108" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>25/08/2026</t>
         </is>
       </c>
       <c r="E42" s="109" t="inlineStr">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="F42" s="109" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G42" s="109" t="inlineStr">
@@ -3230,7 +3234,11 @@
       <c r="I42" s="108" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="109" t="n"/>
+      <c r="J42" s="109" t="inlineStr">
+        <is>
+          <t>21/10/2026 : transcription relue visuellement page par page contre le PDF (6 pages, scan sans texte) et réécrite. Date lue sur la page 5 : « Fait à Angers, le 25/08/2026 ». Seule signature visible : Pr Mario CAMPONE, Directeur Général. Dans le PDF, les pages 5 et 6 sont inversées (le 3-18 continue de la page 6 à la page 5). Tableau du FMD (3-1) et chiffres (449,31 ETP, 1097,23 ETP) corrigés par rapport à l'OCR. Word : en attente de réception.</t>
+        </is>
+      </c>
       <c r="K42" s="109" t="n"/>
       <c r="L42" s="109" t="n"/>
     </row>
@@ -3522,7 +3530,7 @@
       </c>
       <c r="F48" s="97" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G48" s="97" t="inlineStr">
@@ -3570,7 +3578,7 @@
       </c>
       <c r="F49" s="97" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G49" s="97" t="inlineStr">
@@ -3618,7 +3626,7 @@
       </c>
       <c r="F50" s="97" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G50" s="97" t="inlineStr">
@@ -3666,7 +3674,7 @@
       </c>
       <c r="F51" s="103" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>manquant (en attente de réception)</t>
         </is>
       </c>
       <c r="G51" s="103" t="inlineStr">
@@ -4147,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4262,6 +4270,13 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mise à jour du 21/10/2026 : aucun Word reçu pour l'avenant Prime USC, les PV de désaccord NAO 2023 et 2026, ni pour les 4 documents scannés (PEE, avenant restauration, don de jours, charte déconnexion) ; ils restent comptés dans « Word d'origine manquants » (en attente de réception). Le PV NAO 2026 est daté du 25/08/2026 et sa transcription a été relue. À venir : négociation du protocole d'accord préélectoral (PAPE) avec la direction le 22/10/2026 ; le PAPE 2022 est obsolète. Le lien VAP est résolu : le Word « V2025-2 » est celui de l'avenant du 04/02/2025 (le texte du Word dit « le présent avenant »).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A13:B13"/>

</xml_diff>

<commit_message>
Integration des documents du 23/10/2026 : Word, PEE, renommage des Word sans mention plus en vigueur, index corriges
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qy2Wa5ACXajAV16uhKD7cK
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -1252,12 +1252,12 @@
       </c>
       <c r="J5" s="98" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ Signatures CGT-FO et Sud Santé-Sociaux manquantes (seuls DG et CFE-CGC ont signé). ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Signé uniquement par le DG et la CFE-CGC : situation normale, confirmée par David Di Peri le 23/10/2026. ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.</t>
         </is>
       </c>
       <c r="K5" s="98" t="inlineStr">
         <is>
-          <t>Le texte evoque par erreur 'l'amenagement du temps de travail des salaries non-cadre' alors que cet avenant concerne les CADRES (deja signale dans le resume). 'remplacer ... et annuelle' au lieu de 'annule' (faute). Numerotation '4.4 Formalites de depot' alors que la section est '2.1-2.3' (Article 2 -- Dispositions finales) : devrait etre 2.4. Sur le PDF signe, seuls le DG et la CFE-CGC ont signe (CGT-FO et Sud Sante-Sociaux non signataires).</t>
+          <t>Le texte evoque par erreur 'l'amenagement du temps de travail des salaries non-cadre' alors que cet avenant concerne les CADRES (deja signale dans le resume). 'remplacer ... et annuelle' au lieu de 'annule' (faute). Numerotation '4.4 Formalites de depot' alors que la section est '2.1-2.3' (Article 2 -- Dispositions finales) : devrait etre 2.4. Signataires : DG et CFE-CGC (normal, confirmé 23/10/2026).</t>
         </is>
       </c>
       <c r="L5" s="98" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="J8" s="98" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant). ⚠️ ANOMALIE : signature du DG absente (CGT-FO, Sud Santé-Sociaux et CFE-CGC ont signé, pas l'employeur) — à clarifier avec la Direction. Ajouté quand même, signalé clairement (décision David 19/10/2026).</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant). ✅ 23/10/2026 : anomalie levée. David a transmis une autre version scannée du même avenant (texte identique, vérifié par OCR) où le DG (M. Campone) a signé, en plus de CGT-FO, Sud Santé-Sociaux et CFE-CGC (page 5 relue visuellement). PDF du dépôt remplacé par cette version complète.</t>
         </is>
       </c>
       <c r="K8" s="98" t="inlineStr">
@@ -1546,7 +1546,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="100.5" customHeight="1">
+    <row r="11" ht="117.4" customHeight="1">
       <c r="A11" s="95" t="inlineStr">
         <is>
           <t>Compte Épargne Temps (CET)</t>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="F11" s="97" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>Accord CET vDefinitive.docx (reçu le 23/10/2026)</t>
         </is>
       </c>
       <c r="G11" s="97" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="J11" s="97" t="inlineStr">
         <is>
-          <t>PDF de l'accord de base retrouve et integre le 20/10/2026 (David l'a ajoute dans son dossier local). Signatures verifiees visuellement sur le PDF de base (19/03/2021) : ICO (Campone), CGT-FO, CFDT, CFE-CGC ont signe ; Sud Sante-Sociaux (Isabelle Fouillet), partie a l'accord, n'a pas de signature visible sur la page de signature  (même constat pour l'avenant n°1, voir sa ligne). Contenu du .md verifie conforme au PDF signe (preambule, articles 1 a 8, plafonds).</t>
+          <t>PDF de l'accord de base retrouve et integre le 20/10/2026 (David l'a ajoute dans son dossier local). Signatures verifiees visuellement sur le PDF de base (19/03/2021) : ICO (Campone), CGT-FO, CFDT, CFE-CGC ont signe ; Sud Sante-Sociaux (Isabelle Fouillet), partie a l'accord, n'a pas de signature visible sur la page de signature  (même constat pour l'avenant n°1, voir sa ligne). Contenu du .md verifie conforme au PDF signe (preambule, articles 1 a 8, plafonds). 23/10/2026 : Word « vDéfinitive » reçu et rangé, identique au .md (aucun écart de contenu).</t>
         </is>
       </c>
       <c r="K11" s="97" t="inlineStr">
@@ -3050,7 +3050,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
+    <row r="39" ht="54.4" customHeight="1">
       <c r="A39" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2023</t>
@@ -3074,7 +3074,7 @@
       </c>
       <c r="F39" s="109" t="inlineStr">
         <is>
-          <t>manquant (en attente de réception)</t>
+          <t>PV Desaccord NAO 2023.docx (reçu le 23/10/2026)</t>
         </is>
       </c>
       <c r="G39" s="109" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="J39" s="109" t="inlineStr">
         <is>
-          <t>Word en attente de réception (David le recherche).</t>
+          <t>Word reçu le 23/10/2026 et rangé dans le dossier Word NAO. Comparé au .md : identique, sauf « une prime covoiturage » (Word) contre « un prime covoiturage » (md et PDF signé, vérifié visuellement) ; le .md reste fidèle au PDF.</t>
         </is>
       </c>
       <c r="K39" s="109" t="n"/>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="F40" s="109" t="inlineStr">
         <is>
-          <t>PV NAO 2024 - V Finale plus en vigueur.docx</t>
+          <t>PV NAO 2024 V Finale.docx</t>
         </is>
       </c>
       <c r="G40" s="109" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="F41" s="109" t="inlineStr">
         <is>
-          <t>PV NAO 2025 - V 2 plus en vigueur.docx</t>
+          <t>PV NAO 2025 V 2.docx</t>
         </is>
       </c>
       <c r="G41" s="109" t="inlineStr">
@@ -3194,7 +3194,7 @@
       <c r="K41" s="109" t="n"/>
       <c r="L41" s="109" t="n"/>
     </row>
-    <row r="42" ht="33" customHeight="1">
+    <row r="42" ht="142.6" customHeight="1">
       <c r="A42" s="107" t="inlineStr">
         <is>
           <t>PV de désaccord NAO 2026</t>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="F42" s="109" t="inlineStr">
         <is>
-          <t>manquant (en attente de réception)</t>
+          <t>PV NAO 2026 V2.docx (reçu le 23/10/2026)</t>
         </is>
       </c>
       <c r="G42" s="109" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="J42" s="109" t="inlineStr">
         <is>
-          <t>21/10/2026 : transcription relue visuellement page par page contre le PDF (6 pages, scan sans texte) et réécrite. Date lue sur la page 5 : « Fait à Angers, le 25/08/2026 ». Seule signature visible : Pr Mario CAMPONE, Directeur Général. Dans le PDF, les pages 5 et 6 sont inversées (le 3-18 continue de la page 6 à la page 5). Tableau du FMD (3-1) et chiffres (449,31 ETP, 1097,23 ETP) corrigés par rapport à l'OCR. Word : en attente de réception.</t>
+          <t>21/10/2026 : transcription relue visuellement page par page contre le PDF (6 pages, scan sans texte) et réécrite. Date lue sur la page 5 : « Fait à Angers, le 25/08/2026 ». Seule signature visible : Pr Mario CAMPONE, Directeur Général. Dans le PDF, les pages 5 et 6 sont inversées (le 3-18 continue de la page 6 à la page 5). Tableau du FMD (3-1) et chiffres (449,31 ETP, 1097,23 ETP) corrigés par rapport à l'OCR. 23/10/2026 : Word reçu et rangé ; comparé au .md : une erreur d'OCR corrigée (« le soutien scolaire ou l'aide à domicile », vérifié sur le PDF signé page 2). Le PDF porte aussi « l'ancien à accord » (faute du document d'origine), conservée.</t>
         </is>
       </c>
       <c r="K42" s="109" t="n"/>
@@ -3338,7 +3338,7 @@
       <c r="K44" s="94" t="n"/>
       <c r="L44" s="94" t="n"/>
     </row>
-    <row r="45" ht="100.5" customHeight="1">
+    <row r="45" ht="142.6" customHeight="1">
       <c r="A45" s="95" t="inlineStr">
         <is>
           <t>Accord intergénérationnel</t>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="F45" s="97" t="inlineStr">
         <is>
-          <t>manquant</t>
+          <t>Accord Intergenerationnel Version 20200130.docx (reçu le 23/10/2026)</t>
         </is>
       </c>
       <c r="G45" s="97" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="J45" s="97" t="inlineStr">
         <is>
-          <t>Corrigé le 20/10/2026 : l'avenant n°1 (30/06/2021) a été restauré au catalogue (voir ligne dédiée), toujours en vigueur en parallèle de l'avenant 2023 (aucun des deux ne s'abroge expressément). Signataires de l'accord de 2020 (lecture du PDF signé) : CGT-FO, Sud et CFE-CGC ; la CFDT n'a pas signé. ⚠️ Point ouvert : date du 30/01/2020 (clause de signature) contre séance du 3 février 2020 (art. 6.5), voir colonne Coquilles.</t>
+          <t>Corrigé le 20/10/2026 : l'avenant n°1 (30/06/2021) a été restauré au catalogue (voir ligne dédiée), toujours en vigueur en parallèle de l'avenant 2023 (aucun des deux ne s'abroge expressément). Signataires de l'accord de 2020 (lecture du PDF signé) : CGT-FO, Sud et CFE-CGC ; la CFDT n'a pas signé. ⚠️ Point ouvert : date du 30/01/2020 (clause de signature) contre séance du 3 février 2020 (art. 6.5), voir colonne Coquilles. 23/10/2026 : Word de l'accord de base reçu et rangé. Texte conforme au .md ; 14 écarts de forme (fautes de la version Word, ex. « gestion prévisionnel ») : le .md suit le PDF signé et n'est pas modifié. Résumé et dépliant non concernés.</t>
         </is>
       </c>
       <c r="K45" s="97" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="F46" s="98" t="inlineStr">
         <is>
-          <t>Accord Intergénérationnel_Avenant n°1_vDéfinitive plus en vigueur.docx (dossier archive-accords-locaux/Format word ; version de travail définitive avant signature ; le nom du fichier dit « plus en vigueur », à renommer ou à confirmer)</t>
+          <t>Avenant Accord Intergenerationnel n1 vDefinitive.docx (dossier accords locaux/Accords locaux Format word ; version de travail définitive avant signature ; renommé le 23/10/2026, mention « plus en vigueur » retirée du nom)</t>
         </is>
       </c>
       <c r="G46" s="98" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="F47" s="98" t="inlineStr">
         <is>
-          <t>Avenant Accord Intergénérationnel 2023 plus en vigueur.docx (dossier archive-accords-locaux/Format word ; le nom du fichier dit « plus en vigueur », à renommer ou à confirmer)</t>
+          <t>Avenant Accord Intergenerationnel 2023.docx (dossier accords locaux/Accords locaux Format word ; renommé et déplacé le 23/10/2026, mention « plus en vigueur » retirée du nom)</t>
         </is>
       </c>
       <c r="G47" s="98" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="J47" s="98" t="inlineStr">
         <is>
-          <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Modifie l'art. 3.4.2 (temps partiel fin de carrière). Aucun Word reçu. 20/10/2026 : Word retrouvé dans l'archive (non comparé au PDF signé dans cette passe).</t>
+          <t>Nouvelle ligne le 19/10/2026 (séparée de l'accord de base). Modifie l'art. 3.4.2 (temps partiel fin de carrière). Aucun Word reçu. 20/10/2026 : Word retrouvé dans l'archive (non comparé au PDF signé dans cette passe). 23/10/2026 : Word renommé et sorti de l'archive.</t>
         </is>
       </c>
       <c r="K47" s="98" t="inlineStr">
@@ -3506,7 +3506,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="87" customHeight="1">
+    <row r="48" ht="142.6" customHeight="1">
       <c r="A48" s="95" t="inlineStr">
         <is>
           <t>Plan d'Épargne d'Entreprise (PEE)</t>
@@ -3530,17 +3530,17 @@
       </c>
       <c r="F48" s="97" t="inlineStr">
         <is>
-          <t>manquant (en attente de réception)</t>
+          <t>Reglement PEE ICO Version Definitive.docx (reçu le 23/10/2026)</t>
         </is>
       </c>
       <c r="G48" s="97" t="inlineStr">
         <is>
-          <t>resume_PEE_2019.md (dossier en_attente_version_word)</t>
+          <t>resume_PEE_2019.md</t>
         </is>
       </c>
       <c r="H48" s="97" t="inlineStr">
         <is>
-          <t>Depliant_PEE_FO.pdf (dossier en_attente_version_word)</t>
+          <t>Depliant_PEE_FO.pdf</t>
         </is>
       </c>
       <c r="I48" s="96" t="n">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="J48" s="97" t="inlineStr">
         <is>
-          <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG le 22/02/2019 — CGT-FO et CFE-CGC signataires, CGT et Sud Santé-Sociaux non signataires. 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Accord PEE signe par FO et CGC.md ». ⚠️ À vérifier : abondement du PEE.</t>
+          <t>Nouveau le 19/10/2026 (transmis par David, PDF scanné OCR relu visuellement). Signé par le DG le 22/02/2019 — CGT-FO et CFE-CGC signataires, CGT et Sud Santé-Sociaux non signataires. 20/10/2026 : résumé et dépliant produits (dossier en_attente_version_word, en attente d'un Word d'origine) ; Markdown OCR « Accord PEE signe par FO et CGC.md ».  23/10/2026 : Word reçu et rangé ; résumé et dépliant vérifiés contre le Word et mis en production (une correction : « divorce, séparation ou dissolution de Pacs »). Abondement : confirmé sur le Word, l'art. 2 renvoie à l'art. 3 qui ne prévoit que les frais de tenue de compte, aucun montant d'abondement chiffré.</t>
         </is>
       </c>
       <c r="K48" s="97" t="n"/>
@@ -4155,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4165,7 +4165,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Synthèse recalculée le 20 octobre 2026 (une ligne du tableau = un document)</t>
+          <t>Synthèse recalculée le 23 octobre 2026 (une ligne du tableau = un document)</t>
         </is>
       </c>
       <c r="B1" s="14" t="n"/>
@@ -4207,7 +4207,7 @@
         </is>
       </c>
       <c r="B6" s="18" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -4274,6 +4274,13 @@
       <c r="A15" t="inlineStr">
         <is>
           <t>Mise à jour du 21/10/2026 : aucun Word reçu pour l'avenant Prime USC, les PV de désaccord NAO 2023 et 2026, ni pour les 4 documents scannés (PEE, avenant restauration, don de jours, charte déconnexion) ; ils restent comptés dans « Word d'origine manquants » (en attente de réception). Le PV NAO 2026 est daté du 25/08/2026 et sa transcription a été relue. À venir : négociation du protocole d'accord préélectoral (PAPE) avec la direction le 22/10/2026 ; le PAPE 2022 est obsolète. Le lien VAP est résolu : le Word « V2025-2 » est celui de l'avenant du 04/02/2025 (le texte du Word dit « le présent avenant »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mise à jour du 23/10/2026 : 5 Word reçus et rangés (CET base, accord intergénérationnel base, PEE, PV NAO 2023, PV NAO 2026) ; 5 fichiers reçus étaient des doublons exacts de ceux du dépôt (PV NAO 2024, PV NAO 2025, prime USC, VAP, avenant intergénérationnel 2023) ; le PDF de l'avenant ATT non cadres (congés payés) est remplacé par la version signée aussi par le DG. Chiffre « Word manquants » recalculé.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Barres de recherche : indication « je suis IDE » ; Excel de suivi : doute sur les DUE 2022
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ZH9uJbiB7eJrQsuh3THLD
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -3844,7 +3844,7 @@
       </c>
       <c r="J54" s="103" t="inlineStr">
         <is>
-          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes).</t>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Verifie le 28/10/2026 sur le texte : les art. 1 et 2 parlent de frais de sante, mais l'art. 4 fixe des cotisations en pourcentage par tranches du plafond de la Securite sociale (comme les notices de prevoyance AXA) et l'art. 8 traite des rentes d'incapacite et d'invalidite et des garanties deces. La conclusion 'erreur de denomination, regime frais de sante remplace en 2024' n'est donc pas confirmee : a verifier aupres de la Direction avant de la considerer comme historique. Art. 2 de la version cadre : cadres (positions 6 et 7) et fonctions de praticien (PU-PH, MCU-PH, chef de clinique, interne).</t>
         </is>
       </c>
       <c r="K54" s="103" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="J55" s="103" t="inlineStr">
         <is>
-          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Difference avec la version non cadre : perimetre (positions 6-7 CCN + praticiens) et cotisations (3 tranches PASS au lieu de 2, taux differents).</t>
+          <t>Ajoute le 20/10/2026 (transmis par David, dossier local 'Prevoyance, mutuelle, retraite'). Regime en vigueur du 01/07/2022 au 31/05/2024, probablement remplace par la DUE Complementaire Frais de Sante du 19/06/2024 (deduction, non confirmee explicitement par les textes). Difference avec la version non cadre : perimetre (positions 6-7 CCN + praticiens) et cotisations (3 tranches PASS au lieu de 2, taux differents). Verifie le 28/10/2026 sur le texte : les art. 1 et 2 parlent de frais de sante, mais l'art. 4 fixe des cotisations en pourcentage par tranches du plafond de la Securite sociale (comme les notices de prevoyance AXA) et l'art. 8 traite des rentes d'incapacite et d'invalidite et des garanties deces. La conclusion 'erreur de denomination, regime frais de sante remplace en 2024' n'est donc pas confirmee : a verifier aupres de la Direction avant de la considerer comme historique. Art. 2 de la version cadre : cadres (positions 6 et 7) et fonctions de praticien (PU-PH, MCU-PH, chef de clinique, interne).</t>
         </is>
       </c>
       <c r="K55" s="103" t="inlineStr">

</xml_diff>

<commit_message>
Accueil, mentions légales, bandeaux d'avertissement, GitHub retiré, commentaires retirés des résumés et dépliants
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ZH9uJbiB7eJrQsuh3THLD
</commit_message>
<xml_diff>
--- a/Suivi accord ICO.xlsx
+++ b/Suivi accord ICO.xlsx
@@ -1196,7 +1196,8 @@
       </c>
       <c r="J4" s="97" t="inlineStr">
         <is>
-          <t>Avenant congés payés maladie (31/12/2025) désormais sur sa propre ligne, voir 'Avenant — Congés payés...'.</t>
+          <t>Avenant congés payés maladie (31/12/2025) désormais sur sa propre ligne, voir 'Avenant — Congés payés...'.
+29/10/2026 : Retire des résumés et dépliants (commentaires de relecture, à garder ici) : numérotation 1.1.3 à 1.1.5 du texte signé citée telle quelle (le résumé cite l'article 1.3) ; mention « règle en vigueur depuis le 31/12/2025 » et paragraphe sur le changement de règle des congés payés pendant un arrêt maladie ; le texte ne précise pas devant quelle instance le bilan est présenté.</t>
         </is>
       </c>
       <c r="K4" s="97" t="inlineStr">
@@ -1252,7 +1253,8 @@
       </c>
       <c r="J5" s="98" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Signé uniquement par le DG et la CFE-CGC : situation normale, confirmée par David Di Peri le 23/10/2026. ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Signé uniquement par le DG et la CFE-CGC : situation normale, confirmée par David Di Peri le 23/10/2026. ⚠️ Préambule du PDF mentionne par erreur 'non-cadre'.
+29/10/2026 : Retire du résumé : mention « seul point modifié, le reste de l'accord de 2021 est inchangé ».</t>
         </is>
       </c>
       <c r="K5" s="98" t="inlineStr">
@@ -1308,7 +1310,8 @@
       </c>
       <c r="J6" s="97" t="inlineStr">
         <is>
-          <t>Avenant n°1 (CET heures supplémentaires, 31/01/2022) et avenant congés payés maladie (31/12/2025) : voir leurs lignes dédiées (séparées le 20/10/2026). Les deux sont intégrés au résumé.</t>
+          <t>Avenant n°1 (CET heures supplémentaires, 31/01/2022) et avenant congés payés maladie (31/12/2025) : voir leurs lignes dédiées (séparées le 20/10/2026). Les deux sont intégrés au résumé.
+29/10/2026 : Retire des résumés et dépliants : le texte ne précise pas devant quelle instance le bilan est présenté ; mention « inchangé par les avenants 2022 et 2025 » (dépliant Travail de nuit).</t>
         </is>
       </c>
       <c r="K6" s="97" t="inlineStr">
@@ -1644,7 +1647,8 @@
       </c>
       <c r="J12" s="98" t="inlineStr">
         <is>
-          <t>Ligne séparée le 20/10/2026. Annule et remplace l'art. 3.3 (alimentation du CET) de l'accord du 19/03/2021 ; date limite de dépôt des éléments temporels fixée au 15 janvier. Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). Mis à la signature du 31/01 au 11/02/2022. PDF servi par le site mais non listé (lien sur le Thème).</t>
+          <t>Ligne séparée le 20/10/2026. Annule et remplace l'art. 3.3 (alimentation du CET) de l'accord du 19/03/2021 ; date limite de dépôt des éléments temporels fixée au 15 janvier. Signatures relues visuellement sur le PDF (pages 3 et 4) : ICO (M. Campone), CGT-FO, CFDT, CFE-CGC ont signé ; Sud Santé-Sociaux (J. Rosan) n'a pas signé (ligne vide). Mis à la signature du 31/01 au 11/02/2022. PDF servi par le site mais non listé (lien sur le Thème).
+29/10/2026 : Retire du résumé CET : historique du report de la date de dépôt (30 novembre repoussé au 15 janvier).</t>
         </is>
       </c>
       <c r="K12" s="98" t="inlineStr">
@@ -1750,7 +1754,11 @@
       <c r="I14" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="97" t="n"/>
+      <c r="J14" s="97" t="inlineStr">
+        <is>
+          <t>29/10/2026 : Retire du résumé PERCOL : mention « les 4 organisations ont signé ». Le dépliant garde la formulation de l'encadré Source.</t>
+        </is>
+      </c>
       <c r="K14" s="97" t="inlineStr">
         <is>
           <t>Orthographe incoherente du nom d'une signataire dans le meme document : 'Genevieve' (preambule) vs 'Genevieve' sans accent (signatures). DIRECCTE correcte pour sa date (19/03/2021, avant le changement d'avril 2021).</t>
@@ -1960,7 +1968,8 @@
       </c>
       <c r="J18" s="97" t="inlineStr">
         <is>
-          <t>Avenant du 04/02/2025 désormais sur sa propre ligne (voir 'Avenant — VAP'). PDF signe (22/03/2024, 'Accord VAP - V2') verifie visuellement page par page le 20/10/2026 : signe ICO (Pr Campone, DG), CGT-FO (David Di Peri), CFE-CGC (Maxime Bremaud). AUCUNE signature ni paraphe de Sud Sante-Sociaux (Julien Rosan) sur les 5 pages -- ce syndicat n'a pas signe l'accord de base.</t>
+          <t>Avenant du 04/02/2025 désormais sur sa propre ligne (voir 'Avenant — VAP'). PDF signe (22/03/2024, 'Accord VAP - V2') verifie visuellement page par page le 20/10/2026 : signe ICO (Pr Campone, DG), CGT-FO (David Di Peri), CFE-CGC (Maxime Bremaud). AUCUNE signature ni paraphe de Sud Sante-Sociaux (Julien Rosan) sur les 5 pages -- ce syndicat n'a pas signe l'accord de base.
+29/10/2026 : Retire du résumé et du dépliant VAP : phrase sur l'automatisation « depuis plusieurs années » avec le taux de 98 %, paragraphe sur les critères d'évaluation, bloc « Ce qui ne change pas ». Les paliers sont désormais cités avec leurs dates (accord du 22/03/2024, avenant du 04/02/2025).</t>
         </is>
       </c>
       <c r="K18" s="97" t="inlineStr">
@@ -2176,7 +2185,8 @@
       </c>
       <c r="J22" s="97" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant) : daté du 24/10/2025, signé DG/CGT-FO/CFE-CGC. ⚠️ Sud Santé-Sociaux n'a pas signé (ligne vide). 20/10/2026 : doublon du PDF non signé supprimé, le lien du résumé pointe vers « signe.pdf ». Signataires du dépliant : DG, CGT-FO et CFE-CGC.</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant) : daté du 24/10/2025, signé DG/CGT-FO/CFE-CGC. ⚠️ Sud Santé-Sociaux n'a pas signé (ligne vide). 20/10/2026 : doublon du PDF non signé supprimé, le lien du résumé pointe vers « signe.pdf ». Signataires du dépliant : DG, CGT-FO et CFE-CGC.
+29/10/2026 : Retire du résumé : mention « (nouveauté 2025) ».</t>
         </is>
       </c>
       <c r="K22" s="97" t="inlineStr">
@@ -2442,7 +2452,11 @@
       <c r="I27" s="102" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="103" t="n"/>
+      <c r="J27" s="103" t="inlineStr">
+        <is>
+          <t>29/10/2026 : Retire du résumé : commentaire sur le suivi de la décision, remplacé par la seule mention de l'outil Chronos (point 5).</t>
+        </is>
+      </c>
       <c r="K27" s="103" t="inlineStr">
         <is>
           <t>Point 3 : 'Des lors que' -- accent manquant sur 'Des' (orthographe). Ambiguite entre le point 4 (prime applicable aux AS/IDE 'depuis la premiere DUE de fevrier 2023') et le point 6 ('prise a effet du 1er mai 2024') -- pas de distinction claire de la date d'effet selon les categories de personnel.</t>
@@ -2494,7 +2508,11 @@
       <c r="I28" s="96" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="97" t="n"/>
+      <c r="J28" s="97" t="inlineStr">
+        <is>
+          <t>29/10/2026 : Retire du résumé : mention « Pas de signataire CFDT ».</t>
+        </is>
+      </c>
       <c r="K28" s="97" t="inlineStr">
         <is>
           <t>Art. 4.3 : 'DIRECCTE d'Angers' -- anachronisme (accord signe 11/03/2025).</t>
@@ -2924,7 +2942,8 @@
       </c>
       <c r="J36" s="103" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.
+29/10/2026 : Retire du résumé : commentaire sur le suivi de la décision, remplacé par « Mécanisme administratif ».</t>
         </is>
       </c>
       <c r="K36" s="103" t="inlineStr">
@@ -2980,7 +2999,8 @@
       </c>
       <c r="J37" s="103" t="inlineStr">
         <is>
-          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.</t>
+          <t>PDF signé retrouvé le 19/10/2026 (était manquant). Conforme au résumé déjà rédigé, aucun écart.
+29/10/2026 : Retire du résumé : commentaire sur le suivi de la décision, remplacé par « Mécanisme administratif ».</t>
         </is>
       </c>
       <c r="K37" s="103" t="inlineStr">
@@ -3944,7 +3964,8 @@
       </c>
       <c r="J56" s="115" t="inlineStr">
         <is>
-          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604120000Q. Garanties verifiees identiques mot pour mot a la version cadre (comparaison textuelle programmatique page par page) -- seul le perimetre des beneficiaires et le numero de contrat different. Resume unique cadre+non cadre avec clause beneficiaire integree.</t>
+          <t>Ajoute le 20/10/2026 (transmis par David). Contrat AXA n2257604120000Q. Garanties verifiees identiques mot pour mot a la version cadre (comparaison textuelle programmatique page par page) -- seul le perimetre des beneficiaires et le numero de contrat different. Resume unique cadre+non cadre avec clause beneficiaire integree.
+29/10/2026 : Retire du résumé : comparaison page par page des deux notices ; remarque sur les catégories de personnel assurées, que les notices ne définissent pas.</t>
         </is>
       </c>
       <c r="K56" s="115" t="n"/>
@@ -4076,7 +4097,8 @@
       </c>
       <c r="J59" s="119" t="inlineStr">
         <is>
-          <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer. Resume redige et integre le 20/10/2026 sur demande de David : notice d'information des assistances AXA possibles. Erreur corrigee dans le .md source : la condition "aucun membre de la famille a moins de 50 km" ne vise que la presence d'un proche au chevet.</t>
+          <t>Ajoute le 20/10/2026. Contrat AXA n2713840 / convention n7203052, distinct des contrats des notices Prevoyance. David doit d'abord relire le contenu (voir recapitulatif fourni dans la conversation) avant decision d'integration dans un resume public. Indice supplementaire : le document mentionne 'votre attestation de tiers payant sante' pour contacter l'assistance, ce qui suggere un rattachement au regime FRAIS DE SANTE plutot qu'a la Prevoyance, malgre son emplacement dans ce dossier -- a confirmer. Resume redige et integre le 20/10/2026 sur demande de David : notice d'information des assistances AXA possibles. Erreur corrigee dans le .md source : la condition "aucun membre de la famille a moins de 50 km" ne vise que la presence d'un proche au chevet.
+29/10/2026 : Retire du résumé et du dépliant Assistances AXA : « Le document dit seulement « bénéficiaires de la garantie » sans préciser laquelle ». Le texte reprend désormais la notice sans commentaire.</t>
         </is>
       </c>
       <c r="K59" s="119" t="n"/>

</xml_diff>